<commit_message>
uploaded files preparing to test task logic for adult summary form
</commit_message>
<xml_diff>
--- a/forms/contact/person-create.xlsx
+++ b/forms/contact/person-create.xlsx
@@ -13,66 +13,75 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="253">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="274">
   <si>
     <t>type</t>
   </si>
   <si>
+    <t>form_title</t>
+  </si>
+  <si>
+    <t>list_name</t>
+  </si>
+  <si>
     <t>name</t>
   </si>
   <si>
+    <t>form_id</t>
+  </si>
+  <si>
     <t>label::en</t>
   </si>
   <si>
+    <t>version</t>
+  </si>
+  <si>
+    <t>style</t>
+  </si>
+  <si>
+    <t>path</t>
+  </si>
+  <si>
+    <t>default_language</t>
+  </si>
+  <si>
     <t>label::fr</t>
   </si>
   <si>
-    <t>form_title</t>
+    <t>New Person</t>
   </si>
   <si>
     <t>label::cr</t>
   </si>
   <si>
-    <t>form_id</t>
+    <t>contact:person:create</t>
   </si>
   <si>
     <t>required</t>
   </si>
   <si>
-    <t>list_name</t>
-  </si>
-  <si>
     <t>relevant</t>
   </si>
   <si>
-    <t>version</t>
-  </si>
-  <si>
     <t>appearance</t>
   </si>
   <si>
-    <t>style</t>
-  </si>
-  <si>
-    <t>path</t>
-  </si>
-  <si>
-    <t>default_language</t>
-  </si>
-  <si>
     <t>read_only</t>
   </si>
   <si>
-    <t>New Person</t>
-  </si>
-  <si>
     <t>constraint</t>
   </si>
   <si>
+    <t>yes_no</t>
+  </si>
+  <si>
     <t>constraint_message::en</t>
   </si>
   <si>
-    <t>contact:person:create</t>
+    <t>true</t>
+  </si>
+  <si>
+    <t>Yes</t>
   </si>
   <si>
     <t>constraint_message::fr</t>
@@ -81,21 +90,15 @@
     <t>constraint_message::cr</t>
   </si>
   <si>
+    <t>Oui</t>
+  </si>
+  <si>
     <t>calculation</t>
   </si>
   <si>
-    <t>yes_no</t>
-  </si>
-  <si>
     <t>choice_filter</t>
   </si>
   <si>
-    <t>true</t>
-  </si>
-  <si>
-    <t>Yes</t>
-  </si>
-  <si>
     <t>hint::en</t>
   </si>
   <si>
@@ -105,9 +108,6 @@
     <t>hint::cr</t>
   </si>
   <si>
-    <t>Oui</t>
-  </si>
-  <si>
     <t>default</t>
   </si>
   <si>
@@ -138,15 +138,21 @@
     <t>Female</t>
   </si>
   <si>
+    <t>NO_LABEL</t>
+  </si>
+  <si>
     <t>Femme</t>
   </si>
   <si>
-    <t>NO_LABEL</t>
+    <t>data</t>
   </si>
   <si>
     <t>Fi</t>
   </si>
   <si>
+    <t>en</t>
+  </si>
+  <si>
     <t>male</t>
   </si>
   <si>
@@ -159,6 +165,9 @@
     <t>Gason</t>
   </si>
   <si>
+    <t>false()</t>
+  </si>
+  <si>
     <t>boy_girl</t>
   </si>
   <si>
@@ -180,15 +189,15 @@
     <t>Ti gason</t>
   </si>
   <si>
-    <t>false()</t>
-  </si>
-  <si>
     <t>select_dob_method</t>
   </si>
   <si>
     <t>approx</t>
   </si>
   <si>
+    <t>user</t>
+  </si>
+  <si>
     <t>Date of birth unknown</t>
   </si>
   <si>
@@ -198,82 +207,79 @@
     <t>Dat nesans enkoni</t>
   </si>
   <si>
-    <t>data</t>
-  </si>
-  <si>
-    <t>en</t>
-  </si>
-  <si>
     <t>roles</t>
   </si>
   <si>
     <t>program_officer</t>
   </si>
   <si>
+    <t>string</t>
+  </si>
+  <si>
+    <t>contact_id</t>
+  </si>
+  <si>
+    <t>Contact ID of the logged in user</t>
+  </si>
+  <si>
+    <t>Identifiant du contact</t>
+  </si>
+  <si>
     <t>Program Officer</t>
   </si>
   <si>
+    <t>Idantifyan kontak itilizatè a</t>
+  </si>
+  <si>
     <t>Chargé de programme</t>
   </si>
   <si>
-    <t>user</t>
-  </si>
-  <si>
     <t>Ofisye Pwogram nan</t>
   </si>
   <si>
-    <t>string</t>
-  </si>
-  <si>
-    <t>contact_id</t>
+    <t>facility_id</t>
+  </si>
+  <si>
+    <t>Place ID of the logged in user</t>
+  </si>
+  <si>
+    <t>Identifiant du centre</t>
+  </si>
+  <si>
+    <t>Idantifyan sant lan</t>
   </si>
   <si>
     <t>nurse</t>
   </si>
   <si>
-    <t>Contact ID of the logged in user</t>
-  </si>
-  <si>
-    <t>Identifiant du contact</t>
-  </si>
-  <si>
     <t>Nurse</t>
   </si>
   <si>
-    <t>Idantifyan kontak itilizatè a</t>
-  </si>
-  <si>
     <t>Infirmière</t>
   </si>
   <si>
     <t>Enfimyè</t>
   </si>
   <si>
+    <t>Name of the logged in user</t>
+  </si>
+  <si>
+    <t>Nom</t>
+  </si>
+  <si>
+    <t>Non itilizatè a</t>
+  </si>
+  <si>
     <t>che</t>
   </si>
   <si>
     <t>Community Health Entrepreneur</t>
   </si>
   <si>
-    <t>facility_id</t>
-  </si>
-  <si>
-    <t>Place ID of the logged in user</t>
-  </si>
-  <si>
-    <t>Identifiant du centre</t>
-  </si>
-  <si>
-    <t>Idantifyan sant lan</t>
-  </si>
-  <si>
-    <t>Name of the logged in user</t>
-  </si>
-  <si>
-    <t>Nom</t>
-  </si>
-  <si>
-    <t>Non itilizatè a</t>
+    <t>hidden</t>
+  </si>
+  <si>
+    <t>end group</t>
   </si>
   <si>
     <t>Antreprenè Sante Kominotè</t>
@@ -291,9 +297,6 @@
     <t>Sipèvizè Enfimyè</t>
   </si>
   <si>
-    <t>hidden</t>
-  </si>
-  <si>
     <t>patient</t>
   </si>
   <si>
@@ -303,6 +306,9 @@
     <t>Pasyan</t>
   </si>
   <si>
+    <t>init</t>
+  </si>
+  <si>
     <t>other</t>
   </si>
   <si>
@@ -315,6 +321,9 @@
     <t>Lòt</t>
   </si>
   <si>
+    <t>Cannot be inside the person group without having all fields saved to person. And needs separate db-objects because cannot have one that handles the different place types. Last part is now incorrect... as long as it is read only it could be a string of appearance db-object and work fine.</t>
+  </si>
+  <si>
     <t>place_type</t>
   </si>
   <si>
@@ -324,6 +333,27 @@
     <t>Country Department</t>
   </si>
   <si>
+    <t>parent_id</t>
+  </si>
+  <si>
+    <t>Belongs To</t>
+  </si>
+  <si>
+    <t>Associé avec</t>
+  </si>
+  <si>
+    <t>Asosye ak</t>
+  </si>
+  <si>
+    <t>select-contact</t>
+  </si>
+  <si>
+    <t>${parent}</t>
+  </si>
+  <si>
+    <t>${type_label}</t>
+  </si>
+  <si>
     <t>Depatman peyi a</t>
   </si>
   <si>
@@ -333,9 +363,6 @@
     <t>Supervisor Region</t>
   </si>
   <si>
-    <t>end group</t>
-  </si>
-  <si>
     <t>Rejyon sipèvizyon</t>
   </si>
   <si>
@@ -348,31 +375,13 @@
     <t>Zòn enfimyè</t>
   </si>
   <si>
-    <t>init</t>
-  </si>
-  <si>
-    <t>Cannot be inside the person group without having all fields saved to person. And needs separate db-objects because cannot have one that handles the different place types. Last part is now incorrect... as long as it is read only it could be a string of appearance db-object and work fine.</t>
-  </si>
-  <si>
-    <t>parent_id</t>
-  </si>
-  <si>
-    <t>Belongs To</t>
-  </si>
-  <si>
-    <t>Associé avec</t>
-  </si>
-  <si>
-    <t>Asosye ak</t>
-  </si>
-  <si>
-    <t>select-contact</t>
-  </si>
-  <si>
-    <t>${parent}</t>
-  </si>
-  <si>
-    <t>${type_label}</t>
+    <t>chronic_conditions</t>
+  </si>
+  <si>
+    <t>hypertension</t>
+  </si>
+  <si>
+    <t>Hypertension</t>
   </si>
   <si>
     <t>select_one place_type</t>
@@ -381,16 +390,40 @@
     <t>type_selector</t>
   </si>
   <si>
+    <t>diabetes</t>
+  </si>
+  <si>
+    <t>Diabetes</t>
+  </si>
+  <si>
     <t>../type</t>
   </si>
   <si>
+    <t>previous_stroke</t>
+  </si>
+  <si>
+    <t>Previous Stroke</t>
+  </si>
+  <si>
     <t>calculate</t>
   </si>
   <si>
     <t>type_label</t>
   </si>
   <si>
+    <t>asthma</t>
+  </si>
+  <si>
+    <t>Asthma</t>
+  </si>
+  <si>
     <t>jr:choice-name(${type_selector},'${type_selector}')</t>
+  </si>
+  <si>
+    <t>none</t>
+  </si>
+  <si>
+    <t>None of the above</t>
   </si>
   <si>
     <t>person</t>
@@ -722,6 +755,36 @@
   </si>
   <si>
     <t>selected( ${role},'other')</t>
+  </si>
+  <si>
+    <t>select_multiple chronic_conditions</t>
+  </si>
+  <si>
+    <t>**Select all that the person has previously been diagnosed with**</t>
+  </si>
+  <si>
+    <t>chronic_hypertension</t>
+  </si>
+  <si>
+    <t>selected(${chronic_conditions}, 'hypertension')</t>
+  </si>
+  <si>
+    <t>chronic_diabetes</t>
+  </si>
+  <si>
+    <t>selected(${chronic_conditions}, 'diabetes')</t>
+  </si>
+  <si>
+    <t>chronic_stroke</t>
+  </si>
+  <si>
+    <t>selected(${chronic_conditions}, 'previous_stroke')</t>
+  </si>
+  <si>
+    <t>chronic_asthma</t>
+  </si>
+  <si>
+    <t>selected(${chronic_conditions}, 'asthma')</t>
   </si>
   <si>
     <t>external_id</t>
@@ -866,36 +929,37 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="37">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="1" fillId="3" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
+    <xf borderId="1" fillId="3" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
     <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
     <xf borderId="1" fillId="4" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="49" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="1" fillId="5" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
     <xf borderId="1" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="5" fontId="3" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="49" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
@@ -905,7 +969,6 @@
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="5" fontId="3" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
@@ -924,6 +987,9 @@
     <xf borderId="1" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" vertical="bottom"/>
     </xf>
+    <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
     <xf borderId="1" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left"/>
     </xf>
@@ -940,6 +1006,12 @@
     </xf>
     <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="6" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1190,55 +1262,55 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="3" t="s">
         <v>5</v>
       </c>
+      <c r="D1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>12</v>
+      </c>
       <c r="F1" s="1" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="K1" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="K1" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="M1" s="3" t="s">
-        <v>21</v>
+      <c r="L1" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="M1" s="5" t="s">
+        <v>24</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="Q1" s="3" t="s">
         <v>29</v>
+      </c>
+      <c r="R1" s="5" t="s">
+        <v>30</v>
       </c>
       <c r="S1" s="1" t="s">
         <v>31</v>
@@ -1251,266 +1323,266 @@
       <c r="B2" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="C2" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="D2" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="E2" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="F2" s="11"/>
-      <c r="G2" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="H2" s="11"/>
-      <c r="I2" s="11"/>
-      <c r="J2" s="11"/>
-      <c r="K2" s="11"/>
-      <c r="L2" s="11"/>
-      <c r="M2" s="11"/>
-      <c r="N2" s="11"/>
-      <c r="O2" s="11"/>
-      <c r="P2" s="11"/>
-      <c r="Q2" s="11"/>
-      <c r="R2" s="11"/>
-      <c r="S2" s="11"/>
-      <c r="T2" s="11"/>
-      <c r="U2" s="11"/>
-      <c r="V2" s="11"/>
-      <c r="W2" s="11"/>
-      <c r="X2" s="11"/>
-      <c r="Y2" s="11"/>
-      <c r="Z2" s="11"/>
-      <c r="AA2" s="11"/>
-      <c r="AB2" s="11"/>
-      <c r="AC2" s="11"/>
-      <c r="AD2" s="11"/>
-      <c r="AE2" s="11"/>
-      <c r="AF2" s="11"/>
-      <c r="AG2" s="18"/>
-      <c r="AH2" s="18"/>
-      <c r="AI2" s="18"/>
-      <c r="AJ2" s="18"/>
-      <c r="AK2" s="18"/>
-      <c r="AL2" s="18"/>
+      <c r="C2" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="D2" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="E2" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="12"/>
+      <c r="K2" s="12"/>
+      <c r="L2" s="12"/>
+      <c r="M2" s="12"/>
+      <c r="N2" s="12"/>
+      <c r="O2" s="12"/>
+      <c r="P2" s="12"/>
+      <c r="Q2" s="12"/>
+      <c r="R2" s="12"/>
+      <c r="S2" s="12"/>
+      <c r="T2" s="12"/>
+      <c r="U2" s="12"/>
+      <c r="V2" s="12"/>
+      <c r="W2" s="12"/>
+      <c r="X2" s="12"/>
+      <c r="Y2" s="12"/>
+      <c r="Z2" s="12"/>
+      <c r="AA2" s="12"/>
+      <c r="AB2" s="12"/>
+      <c r="AC2" s="12"/>
+      <c r="AD2" s="12"/>
+      <c r="AE2" s="12"/>
+      <c r="AF2" s="12"/>
+      <c r="AG2" s="14"/>
+      <c r="AH2" s="14"/>
+      <c r="AI2" s="14"/>
+      <c r="AJ2" s="14"/>
+      <c r="AK2" s="14"/>
+      <c r="AL2" s="14"/>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="10" t="s">
         <v>33</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="C3" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="D3" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="E3" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="F3" s="11"/>
-      <c r="G3" s="11"/>
-      <c r="H3" s="11"/>
-      <c r="I3" s="11"/>
-      <c r="J3" s="11"/>
-      <c r="K3" s="11"/>
-      <c r="L3" s="11"/>
-      <c r="M3" s="11"/>
-      <c r="N3" s="11"/>
-      <c r="O3" s="11"/>
-      <c r="P3" s="11"/>
-      <c r="Q3" s="11"/>
-      <c r="R3" s="11"/>
-      <c r="S3" s="11"/>
-      <c r="T3" s="11"/>
-      <c r="U3" s="11"/>
-      <c r="V3" s="11"/>
-      <c r="W3" s="11"/>
-      <c r="X3" s="11"/>
-      <c r="Y3" s="11"/>
-      <c r="Z3" s="11"/>
-      <c r="AA3" s="11"/>
-      <c r="AB3" s="11"/>
-      <c r="AC3" s="11"/>
-      <c r="AD3" s="11"/>
-      <c r="AE3" s="11"/>
-      <c r="AF3" s="11"/>
-      <c r="AG3" s="18"/>
-      <c r="AH3" s="18"/>
-      <c r="AI3" s="18"/>
-      <c r="AJ3" s="18"/>
-      <c r="AK3" s="18"/>
-      <c r="AL3" s="18"/>
+        <v>60</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="E3" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="F3" s="12"/>
+      <c r="G3" s="12"/>
+      <c r="H3" s="12"/>
+      <c r="I3" s="12"/>
+      <c r="J3" s="12"/>
+      <c r="K3" s="12"/>
+      <c r="L3" s="12"/>
+      <c r="M3" s="12"/>
+      <c r="N3" s="12"/>
+      <c r="O3" s="12"/>
+      <c r="P3" s="12"/>
+      <c r="Q3" s="12"/>
+      <c r="R3" s="12"/>
+      <c r="S3" s="12"/>
+      <c r="T3" s="12"/>
+      <c r="U3" s="12"/>
+      <c r="V3" s="12"/>
+      <c r="W3" s="12"/>
+      <c r="X3" s="12"/>
+      <c r="Y3" s="12"/>
+      <c r="Z3" s="12"/>
+      <c r="AA3" s="12"/>
+      <c r="AB3" s="12"/>
+      <c r="AC3" s="12"/>
+      <c r="AD3" s="12"/>
+      <c r="AE3" s="12"/>
+      <c r="AF3" s="12"/>
+      <c r="AG3" s="14"/>
+      <c r="AH3" s="14"/>
+      <c r="AI3" s="14"/>
+      <c r="AJ3" s="14"/>
+      <c r="AK3" s="14"/>
+      <c r="AL3" s="14"/>
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="D4" s="13" t="s">
         <v>69</v>
       </c>
-      <c r="B4" s="10" t="s">
-        <v>70</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="D4" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="E4" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F4" s="11"/>
-      <c r="G4" s="11"/>
-      <c r="H4" s="11"/>
-      <c r="I4" s="11"/>
-      <c r="J4" s="11"/>
-      <c r="K4" s="11"/>
-      <c r="L4" s="11"/>
-      <c r="M4" s="11"/>
-      <c r="N4" s="11"/>
-      <c r="O4" s="11"/>
-      <c r="P4" s="11"/>
-      <c r="Q4" s="11"/>
-      <c r="R4" s="11"/>
-      <c r="S4" s="11"/>
-      <c r="T4" s="11"/>
-      <c r="U4" s="11"/>
-      <c r="V4" s="11"/>
-      <c r="W4" s="11"/>
-      <c r="X4" s="11"/>
-      <c r="Y4" s="11"/>
-      <c r="Z4" s="11"/>
-      <c r="AA4" s="11"/>
-      <c r="AB4" s="11"/>
-      <c r="AC4" s="11"/>
-      <c r="AD4" s="11"/>
-      <c r="AE4" s="11"/>
-      <c r="AF4" s="11"/>
-      <c r="AG4" s="18"/>
-      <c r="AH4" s="18"/>
-      <c r="AI4" s="18"/>
-      <c r="AJ4" s="18"/>
-      <c r="AK4" s="18"/>
-      <c r="AL4" s="18"/>
+      <c r="E4" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="F4" s="12"/>
+      <c r="G4" s="12"/>
+      <c r="H4" s="12"/>
+      <c r="I4" s="12"/>
+      <c r="J4" s="12"/>
+      <c r="K4" s="12"/>
+      <c r="L4" s="12"/>
+      <c r="M4" s="12"/>
+      <c r="N4" s="12"/>
+      <c r="O4" s="12"/>
+      <c r="P4" s="12"/>
+      <c r="Q4" s="12"/>
+      <c r="R4" s="12"/>
+      <c r="S4" s="12"/>
+      <c r="T4" s="12"/>
+      <c r="U4" s="12"/>
+      <c r="V4" s="12"/>
+      <c r="W4" s="12"/>
+      <c r="X4" s="12"/>
+      <c r="Y4" s="12"/>
+      <c r="Z4" s="12"/>
+      <c r="AA4" s="12"/>
+      <c r="AB4" s="12"/>
+      <c r="AC4" s="12"/>
+      <c r="AD4" s="12"/>
+      <c r="AE4" s="12"/>
+      <c r="AF4" s="12"/>
+      <c r="AG4" s="14"/>
+      <c r="AH4" s="14"/>
+      <c r="AI4" s="14"/>
+      <c r="AJ4" s="14"/>
+      <c r="AK4" s="14"/>
+      <c r="AL4" s="14"/>
     </row>
     <row r="5" ht="14.25" customHeight="1">
       <c r="A5" s="10" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>80</v>
-      </c>
-      <c r="C5" s="11" t="s">
-        <v>81</v>
-      </c>
-      <c r="D5" s="12" t="s">
-        <v>82</v>
-      </c>
-      <c r="E5" s="12" t="s">
-        <v>83</v>
-      </c>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
-      <c r="H5" s="11"/>
-      <c r="I5" s="11"/>
-      <c r="J5" s="11"/>
-      <c r="K5" s="11"/>
-      <c r="L5" s="11"/>
-      <c r="M5" s="11"/>
-      <c r="N5" s="11"/>
-      <c r="O5" s="11"/>
-      <c r="P5" s="11"/>
-      <c r="Q5" s="11"/>
-      <c r="R5" s="11"/>
-      <c r="S5" s="11"/>
-      <c r="T5" s="11"/>
-      <c r="U5" s="11"/>
-      <c r="V5" s="11"/>
-      <c r="W5" s="11"/>
-      <c r="X5" s="11"/>
-      <c r="Y5" s="11"/>
-      <c r="Z5" s="11"/>
-      <c r="AA5" s="11"/>
-      <c r="AB5" s="11"/>
-      <c r="AC5" s="11"/>
-      <c r="AD5" s="11"/>
-      <c r="AE5" s="11"/>
-      <c r="AF5" s="11"/>
-      <c r="AG5" s="18"/>
-      <c r="AH5" s="18"/>
-      <c r="AI5" s="18"/>
-      <c r="AJ5" s="18"/>
-      <c r="AK5" s="18"/>
-      <c r="AL5" s="18"/>
+        <v>74</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="F5" s="12"/>
+      <c r="G5" s="12"/>
+      <c r="H5" s="12"/>
+      <c r="I5" s="12"/>
+      <c r="J5" s="12"/>
+      <c r="K5" s="12"/>
+      <c r="L5" s="12"/>
+      <c r="M5" s="12"/>
+      <c r="N5" s="12"/>
+      <c r="O5" s="12"/>
+      <c r="P5" s="12"/>
+      <c r="Q5" s="12"/>
+      <c r="R5" s="12"/>
+      <c r="S5" s="12"/>
+      <c r="T5" s="12"/>
+      <c r="U5" s="12"/>
+      <c r="V5" s="12"/>
+      <c r="W5" s="12"/>
+      <c r="X5" s="12"/>
+      <c r="Y5" s="12"/>
+      <c r="Z5" s="12"/>
+      <c r="AA5" s="12"/>
+      <c r="AB5" s="12"/>
+      <c r="AC5" s="12"/>
+      <c r="AD5" s="12"/>
+      <c r="AE5" s="12"/>
+      <c r="AF5" s="12"/>
+      <c r="AG5" s="14"/>
+      <c r="AH5" s="14"/>
+      <c r="AI5" s="14"/>
+      <c r="AJ5" s="14"/>
+      <c r="AK5" s="14"/>
+      <c r="AL5" s="14"/>
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="10" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="C6" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="D6" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="E6" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="D6" s="12" t="s">
-        <v>85</v>
-      </c>
-      <c r="E6" s="12" t="s">
-        <v>86</v>
-      </c>
-      <c r="F6" s="11"/>
-      <c r="G6" s="11"/>
-      <c r="H6" s="11"/>
-      <c r="I6" s="11"/>
-      <c r="J6" s="11"/>
-      <c r="K6" s="11"/>
-      <c r="L6" s="11"/>
-      <c r="M6" s="11"/>
-      <c r="N6" s="11"/>
-      <c r="O6" s="11"/>
-      <c r="P6" s="11"/>
-      <c r="Q6" s="11"/>
-      <c r="R6" s="11"/>
-      <c r="S6" s="11"/>
-      <c r="T6" s="11"/>
-      <c r="U6" s="11"/>
-      <c r="V6" s="11"/>
-      <c r="W6" s="11"/>
-      <c r="X6" s="11"/>
-      <c r="Y6" s="11"/>
-      <c r="Z6" s="11"/>
-      <c r="AA6" s="11"/>
-      <c r="AB6" s="11"/>
-      <c r="AC6" s="11"/>
-      <c r="AD6" s="11"/>
-      <c r="AE6" s="11"/>
-      <c r="AF6" s="11"/>
-      <c r="AG6" s="18"/>
-      <c r="AH6" s="18"/>
-      <c r="AI6" s="18"/>
-      <c r="AJ6" s="18"/>
-      <c r="AK6" s="18"/>
-      <c r="AL6" s="18"/>
+      <c r="F6" s="12"/>
+      <c r="G6" s="12"/>
+      <c r="H6" s="12"/>
+      <c r="I6" s="12"/>
+      <c r="J6" s="12"/>
+      <c r="K6" s="12"/>
+      <c r="L6" s="12"/>
+      <c r="M6" s="12"/>
+      <c r="N6" s="12"/>
+      <c r="O6" s="12"/>
+      <c r="P6" s="12"/>
+      <c r="Q6" s="12"/>
+      <c r="R6" s="12"/>
+      <c r="S6" s="12"/>
+      <c r="T6" s="12"/>
+      <c r="U6" s="12"/>
+      <c r="V6" s="12"/>
+      <c r="W6" s="12"/>
+      <c r="X6" s="12"/>
+      <c r="Y6" s="12"/>
+      <c r="Z6" s="12"/>
+      <c r="AA6" s="12"/>
+      <c r="AB6" s="12"/>
+      <c r="AC6" s="12"/>
+      <c r="AD6" s="12"/>
+      <c r="AE6" s="12"/>
+      <c r="AF6" s="12"/>
+      <c r="AG6" s="14"/>
+      <c r="AH6" s="14"/>
+      <c r="AI6" s="14"/>
+      <c r="AJ6" s="14"/>
+      <c r="AK6" s="14"/>
+      <c r="AL6" s="14"/>
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="22" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D7" s="24" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E7" s="24" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F7" s="23"/>
       <c r="G7" s="23"/>
@@ -1548,472 +1620,472 @@
     </row>
     <row r="8" ht="14.25" customHeight="1">
       <c r="A8" s="10" t="s">
-        <v>106</v>
+        <v>88</v>
       </c>
       <c r="B8" s="10"/>
-      <c r="C8" s="11"/>
-      <c r="D8" s="11"/>
-      <c r="E8" s="11"/>
-      <c r="F8" s="11"/>
-      <c r="G8" s="11"/>
-      <c r="H8" s="11"/>
-      <c r="I8" s="11"/>
-      <c r="J8" s="11"/>
-      <c r="K8" s="11"/>
-      <c r="L8" s="11"/>
-      <c r="M8" s="11"/>
-      <c r="N8" s="11"/>
-      <c r="O8" s="11"/>
-      <c r="P8" s="11"/>
-      <c r="Q8" s="11"/>
-      <c r="R8" s="11"/>
-      <c r="S8" s="11"/>
-      <c r="T8" s="11"/>
-      <c r="U8" s="11"/>
-      <c r="V8" s="11"/>
-      <c r="W8" s="11"/>
-      <c r="X8" s="11"/>
-      <c r="Y8" s="11"/>
-      <c r="Z8" s="11"/>
-      <c r="AA8" s="11"/>
-      <c r="AB8" s="11"/>
-      <c r="AC8" s="11"/>
-      <c r="AD8" s="11"/>
-      <c r="AE8" s="11"/>
-      <c r="AF8" s="11"/>
-      <c r="AG8" s="18"/>
-      <c r="AH8" s="18"/>
-      <c r="AI8" s="18"/>
-      <c r="AJ8" s="18"/>
-      <c r="AK8" s="18"/>
-      <c r="AL8" s="18"/>
+      <c r="C8" s="12"/>
+      <c r="D8" s="12"/>
+      <c r="E8" s="12"/>
+      <c r="F8" s="12"/>
+      <c r="G8" s="12"/>
+      <c r="H8" s="12"/>
+      <c r="I8" s="12"/>
+      <c r="J8" s="12"/>
+      <c r="K8" s="12"/>
+      <c r="L8" s="12"/>
+      <c r="M8" s="12"/>
+      <c r="N8" s="12"/>
+      <c r="O8" s="12"/>
+      <c r="P8" s="12"/>
+      <c r="Q8" s="12"/>
+      <c r="R8" s="12"/>
+      <c r="S8" s="12"/>
+      <c r="T8" s="12"/>
+      <c r="U8" s="12"/>
+      <c r="V8" s="12"/>
+      <c r="W8" s="12"/>
+      <c r="X8" s="12"/>
+      <c r="Y8" s="12"/>
+      <c r="Z8" s="12"/>
+      <c r="AA8" s="12"/>
+      <c r="AB8" s="12"/>
+      <c r="AC8" s="12"/>
+      <c r="AD8" s="12"/>
+      <c r="AE8" s="12"/>
+      <c r="AF8" s="12"/>
+      <c r="AG8" s="14"/>
+      <c r="AH8" s="14"/>
+      <c r="AI8" s="14"/>
+      <c r="AJ8" s="14"/>
+      <c r="AK8" s="14"/>
+      <c r="AL8" s="14"/>
     </row>
     <row r="9" ht="14.25" customHeight="1">
       <c r="A9" s="10" t="s">
-        <v>106</v>
+        <v>88</v>
       </c>
       <c r="B9" s="10"/>
-      <c r="C9" s="11"/>
-      <c r="D9" s="11"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="11"/>
-      <c r="G9" s="11"/>
-      <c r="H9" s="11"/>
-      <c r="I9" s="11"/>
-      <c r="J9" s="11"/>
-      <c r="K9" s="11"/>
-      <c r="L9" s="11"/>
-      <c r="M9" s="11"/>
-      <c r="N9" s="11"/>
-      <c r="O9" s="11"/>
-      <c r="P9" s="11"/>
-      <c r="Q9" s="11"/>
-      <c r="R9" s="11"/>
-      <c r="S9" s="11"/>
-      <c r="T9" s="11"/>
-      <c r="U9" s="11"/>
-      <c r="V9" s="11"/>
-      <c r="W9" s="11"/>
-      <c r="X9" s="11"/>
-      <c r="Y9" s="11"/>
-      <c r="Z9" s="11"/>
-      <c r="AA9" s="11"/>
-      <c r="AB9" s="11"/>
-      <c r="AC9" s="11"/>
-      <c r="AD9" s="11"/>
-      <c r="AE9" s="11"/>
-      <c r="AF9" s="11"/>
-      <c r="AG9" s="18"/>
-      <c r="AH9" s="18"/>
-      <c r="AI9" s="18"/>
-      <c r="AJ9" s="18"/>
-      <c r="AK9" s="18"/>
-      <c r="AL9" s="18"/>
+      <c r="C9" s="12"/>
+      <c r="D9" s="12"/>
+      <c r="E9" s="12"/>
+      <c r="F9" s="12"/>
+      <c r="G9" s="12"/>
+      <c r="H9" s="12"/>
+      <c r="I9" s="12"/>
+      <c r="J9" s="12"/>
+      <c r="K9" s="12"/>
+      <c r="L9" s="12"/>
+      <c r="M9" s="12"/>
+      <c r="N9" s="12"/>
+      <c r="O9" s="12"/>
+      <c r="P9" s="12"/>
+      <c r="Q9" s="12"/>
+      <c r="R9" s="12"/>
+      <c r="S9" s="12"/>
+      <c r="T9" s="12"/>
+      <c r="U9" s="12"/>
+      <c r="V9" s="12"/>
+      <c r="W9" s="12"/>
+      <c r="X9" s="12"/>
+      <c r="Y9" s="12"/>
+      <c r="Z9" s="12"/>
+      <c r="AA9" s="12"/>
+      <c r="AB9" s="12"/>
+      <c r="AC9" s="12"/>
+      <c r="AD9" s="12"/>
+      <c r="AE9" s="12"/>
+      <c r="AF9" s="12"/>
+      <c r="AG9" s="14"/>
+      <c r="AH9" s="14"/>
+      <c r="AI9" s="14"/>
+      <c r="AJ9" s="14"/>
+      <c r="AK9" s="14"/>
+      <c r="AL9" s="14"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="10" t="s">
         <v>33</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>111</v>
-      </c>
-      <c r="C10" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="D10" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="E10" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="F10" s="11"/>
-      <c r="G10" s="11"/>
-      <c r="H10" s="11"/>
-      <c r="I10" s="11"/>
-      <c r="J10" s="11"/>
-      <c r="K10" s="11"/>
-      <c r="L10" s="11"/>
-      <c r="M10" s="11"/>
-      <c r="N10" s="11"/>
-      <c r="O10" s="11"/>
-      <c r="P10" s="11"/>
-      <c r="Q10" s="11"/>
-      <c r="R10" s="11"/>
-      <c r="S10" s="11"/>
-      <c r="T10" s="11"/>
-      <c r="U10" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="V10" s="11"/>
-      <c r="W10" s="11"/>
-      <c r="X10" s="11"/>
-      <c r="Y10" s="11"/>
-      <c r="Z10" s="11"/>
-      <c r="AA10" s="11"/>
-      <c r="AB10" s="11"/>
-      <c r="AC10" s="11"/>
-      <c r="AD10" s="11"/>
-      <c r="AE10" s="11"/>
-      <c r="AF10" s="11"/>
-      <c r="AG10" s="18"/>
-      <c r="AH10" s="18"/>
-      <c r="AI10" s="18"/>
-      <c r="AJ10" s="18"/>
-      <c r="AK10" s="18"/>
-      <c r="AL10" s="18"/>
+        <v>97</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="D10" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="E10" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="F10" s="12"/>
+      <c r="G10" s="12"/>
+      <c r="H10" s="12"/>
+      <c r="I10" s="12"/>
+      <c r="J10" s="12"/>
+      <c r="K10" s="12"/>
+      <c r="L10" s="12"/>
+      <c r="M10" s="12"/>
+      <c r="N10" s="12"/>
+      <c r="O10" s="12"/>
+      <c r="P10" s="12"/>
+      <c r="Q10" s="12"/>
+      <c r="R10" s="12"/>
+      <c r="S10" s="12"/>
+      <c r="T10" s="12"/>
+      <c r="U10" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="V10" s="12"/>
+      <c r="W10" s="12"/>
+      <c r="X10" s="12"/>
+      <c r="Y10" s="12"/>
+      <c r="Z10" s="12"/>
+      <c r="AA10" s="12"/>
+      <c r="AB10" s="12"/>
+      <c r="AC10" s="12"/>
+      <c r="AD10" s="12"/>
+      <c r="AE10" s="12"/>
+      <c r="AF10" s="12"/>
+      <c r="AG10" s="14"/>
+      <c r="AH10" s="14"/>
+      <c r="AI10" s="14"/>
+      <c r="AJ10" s="14"/>
+      <c r="AK10" s="14"/>
+      <c r="AL10" s="14"/>
     </row>
     <row r="11" ht="14.25" customHeight="1">
       <c r="A11" s="10" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>113</v>
-      </c>
-      <c r="C11" s="11" t="s">
-        <v>114</v>
-      </c>
-      <c r="D11" s="12" t="s">
-        <v>115</v>
-      </c>
-      <c r="E11" s="12" t="s">
-        <v>116</v>
-      </c>
-      <c r="F11" s="11"/>
-      <c r="G11" s="11"/>
-      <c r="H11" s="11" t="s">
-        <v>117</v>
-      </c>
-      <c r="I11" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="J11" s="11"/>
-      <c r="K11" s="11"/>
-      <c r="L11" s="11"/>
-      <c r="M11" s="11"/>
-      <c r="N11" s="11" t="s">
-        <v>118</v>
-      </c>
-      <c r="O11" s="11"/>
-      <c r="P11" s="11" t="s">
-        <v>119</v>
-      </c>
-      <c r="Q11" s="12" t="s">
-        <v>119</v>
-      </c>
-      <c r="R11" s="12" t="s">
-        <v>119</v>
-      </c>
-      <c r="S11" s="11"/>
-      <c r="T11" s="11"/>
-      <c r="U11" s="11"/>
-      <c r="V11" s="11"/>
-      <c r="W11" s="11"/>
-      <c r="X11" s="11"/>
-      <c r="Y11" s="11"/>
-      <c r="Z11" s="11"/>
-      <c r="AA11" s="11"/>
-      <c r="AB11" s="11"/>
-      <c r="AC11" s="11"/>
-      <c r="AD11" s="11"/>
-      <c r="AE11" s="11"/>
-      <c r="AF11" s="11"/>
-      <c r="AG11" s="18"/>
-      <c r="AH11" s="18"/>
-      <c r="AI11" s="18"/>
-      <c r="AJ11" s="18"/>
-      <c r="AK11" s="18"/>
-      <c r="AL11" s="18"/>
+        <v>106</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="D11" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="E11" s="13" t="s">
+        <v>109</v>
+      </c>
+      <c r="F11" s="12"/>
+      <c r="G11" s="12"/>
+      <c r="H11" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="I11" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="J11" s="12"/>
+      <c r="K11" s="12"/>
+      <c r="L11" s="12"/>
+      <c r="M11" s="12"/>
+      <c r="N11" s="12" t="s">
+        <v>111</v>
+      </c>
+      <c r="O11" s="12"/>
+      <c r="P11" s="12" t="s">
+        <v>112</v>
+      </c>
+      <c r="Q11" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="R11" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="S11" s="12"/>
+      <c r="T11" s="12"/>
+      <c r="U11" s="12"/>
+      <c r="V11" s="12"/>
+      <c r="W11" s="12"/>
+      <c r="X11" s="12"/>
+      <c r="Y11" s="12"/>
+      <c r="Z11" s="12"/>
+      <c r="AA11" s="12"/>
+      <c r="AB11" s="12"/>
+      <c r="AC11" s="12"/>
+      <c r="AD11" s="12"/>
+      <c r="AE11" s="12"/>
+      <c r="AF11" s="12"/>
+      <c r="AG11" s="14"/>
+      <c r="AH11" s="14"/>
+      <c r="AI11" s="14"/>
+      <c r="AJ11" s="14"/>
+      <c r="AK11" s="14"/>
+      <c r="AL11" s="14"/>
     </row>
     <row r="12" ht="14.25" customHeight="1">
       <c r="A12" s="10" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="C12" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="D12" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="E12" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="F12" s="11"/>
-      <c r="G12" s="11"/>
-      <c r="H12" s="11" t="s">
-        <v>92</v>
-      </c>
-      <c r="I12" s="11"/>
-      <c r="J12" s="11"/>
-      <c r="K12" s="11"/>
-      <c r="L12" s="11"/>
-      <c r="M12" s="11"/>
-      <c r="N12" s="11"/>
-      <c r="O12" s="11"/>
-      <c r="P12" s="11"/>
-      <c r="Q12" s="11"/>
-      <c r="R12" s="11"/>
-      <c r="S12" s="11"/>
-      <c r="T12" s="11"/>
-      <c r="U12" s="11"/>
-      <c r="V12" s="11"/>
-      <c r="W12" s="11"/>
-      <c r="X12" s="11"/>
-      <c r="Y12" s="11"/>
-      <c r="Z12" s="11"/>
-      <c r="AA12" s="11"/>
-      <c r="AB12" s="11"/>
-      <c r="AC12" s="11"/>
-      <c r="AD12" s="11"/>
-      <c r="AE12" s="11"/>
-      <c r="AF12" s="11"/>
-      <c r="AG12" s="18"/>
-      <c r="AH12" s="18"/>
-      <c r="AI12" s="18"/>
-      <c r="AJ12" s="18"/>
-      <c r="AK12" s="18"/>
-      <c r="AL12" s="18"/>
+        <v>3</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="D12" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="E12" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="F12" s="12"/>
+      <c r="G12" s="12"/>
+      <c r="H12" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="I12" s="12"/>
+      <c r="J12" s="12"/>
+      <c r="K12" s="12"/>
+      <c r="L12" s="12"/>
+      <c r="M12" s="12"/>
+      <c r="N12" s="12"/>
+      <c r="O12" s="12"/>
+      <c r="P12" s="12"/>
+      <c r="Q12" s="12"/>
+      <c r="R12" s="12"/>
+      <c r="S12" s="12"/>
+      <c r="T12" s="12"/>
+      <c r="U12" s="12"/>
+      <c r="V12" s="12"/>
+      <c r="W12" s="12"/>
+      <c r="X12" s="12"/>
+      <c r="Y12" s="12"/>
+      <c r="Z12" s="12"/>
+      <c r="AA12" s="12"/>
+      <c r="AB12" s="12"/>
+      <c r="AC12" s="12"/>
+      <c r="AD12" s="12"/>
+      <c r="AE12" s="12"/>
+      <c r="AF12" s="12"/>
+      <c r="AG12" s="14"/>
+      <c r="AH12" s="14"/>
+      <c r="AI12" s="14"/>
+      <c r="AJ12" s="14"/>
+      <c r="AK12" s="14"/>
+      <c r="AL12" s="14"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="10" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C13" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="D13" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="E13" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="F13" s="11"/>
-      <c r="G13" s="11"/>
-      <c r="H13" s="11" t="s">
-        <v>92</v>
-      </c>
-      <c r="I13" s="11"/>
-      <c r="J13" s="11"/>
-      <c r="K13" s="11"/>
-      <c r="L13" s="11"/>
-      <c r="M13" s="11"/>
-      <c r="N13" s="11"/>
-      <c r="O13" s="11"/>
-      <c r="P13" s="11"/>
-      <c r="Q13" s="11"/>
-      <c r="R13" s="11"/>
-      <c r="S13" s="11"/>
-      <c r="T13" s="11"/>
-      <c r="U13" s="11"/>
-      <c r="V13" s="11"/>
-      <c r="W13" s="11"/>
-      <c r="X13" s="11"/>
-      <c r="Y13" s="11"/>
-      <c r="Z13" s="11"/>
-      <c r="AA13" s="11"/>
-      <c r="AB13" s="11"/>
-      <c r="AC13" s="11"/>
-      <c r="AD13" s="11"/>
-      <c r="AE13" s="11"/>
-      <c r="AF13" s="11"/>
-      <c r="AG13" s="18"/>
-      <c r="AH13" s="18"/>
-      <c r="AI13" s="18"/>
-      <c r="AJ13" s="18"/>
-      <c r="AK13" s="18"/>
-      <c r="AL13" s="18"/>
+      <c r="C13" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="D13" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="E13" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="F13" s="12"/>
+      <c r="G13" s="12"/>
+      <c r="H13" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="I13" s="12"/>
+      <c r="J13" s="12"/>
+      <c r="K13" s="12"/>
+      <c r="L13" s="12"/>
+      <c r="M13" s="12"/>
+      <c r="N13" s="12"/>
+      <c r="O13" s="12"/>
+      <c r="P13" s="12"/>
+      <c r="Q13" s="12"/>
+      <c r="R13" s="12"/>
+      <c r="S13" s="12"/>
+      <c r="T13" s="12"/>
+      <c r="U13" s="12"/>
+      <c r="V13" s="12"/>
+      <c r="W13" s="12"/>
+      <c r="X13" s="12"/>
+      <c r="Y13" s="12"/>
+      <c r="Z13" s="12"/>
+      <c r="AA13" s="12"/>
+      <c r="AB13" s="12"/>
+      <c r="AC13" s="12"/>
+      <c r="AD13" s="12"/>
+      <c r="AE13" s="12"/>
+      <c r="AF13" s="12"/>
+      <c r="AG13" s="14"/>
+      <c r="AH13" s="14"/>
+      <c r="AI13" s="14"/>
+      <c r="AJ13" s="14"/>
+      <c r="AK13" s="14"/>
+      <c r="AL13" s="14"/>
     </row>
     <row r="14" ht="14.25" customHeight="1">
       <c r="A14" s="10" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>121</v>
-      </c>
-      <c r="C14" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="D14" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="E14" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="F14" s="11"/>
-      <c r="G14" s="11"/>
-      <c r="H14" s="11" t="s">
-        <v>92</v>
-      </c>
-      <c r="I14" s="11"/>
-      <c r="J14" s="11"/>
-      <c r="K14" s="11"/>
-      <c r="L14" s="11"/>
-      <c r="M14" s="11"/>
-      <c r="N14" s="25" t="s">
-        <v>122</v>
-      </c>
-      <c r="O14" s="11"/>
-      <c r="P14" s="11"/>
-      <c r="Q14" s="11"/>
-      <c r="R14" s="11"/>
-      <c r="S14" s="11"/>
-      <c r="T14" s="11"/>
-      <c r="U14" s="11"/>
-      <c r="V14" s="11"/>
-      <c r="W14" s="11"/>
-      <c r="X14" s="11"/>
-      <c r="Y14" s="11"/>
-      <c r="Z14" s="11"/>
-      <c r="AA14" s="11"/>
-      <c r="AB14" s="11"/>
-      <c r="AC14" s="11"/>
-      <c r="AD14" s="11"/>
-      <c r="AE14" s="11"/>
-      <c r="AF14" s="11"/>
-      <c r="AG14" s="18"/>
-      <c r="AH14" s="18"/>
-      <c r="AI14" s="18"/>
-      <c r="AJ14" s="18"/>
-      <c r="AK14" s="18"/>
-      <c r="AL14" s="18"/>
+        <v>124</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="D14" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="E14" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="F14" s="12"/>
+      <c r="G14" s="12"/>
+      <c r="H14" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="I14" s="12"/>
+      <c r="J14" s="12"/>
+      <c r="K14" s="12"/>
+      <c r="L14" s="12"/>
+      <c r="M14" s="12"/>
+      <c r="N14" s="26" t="s">
+        <v>127</v>
+      </c>
+      <c r="O14" s="12"/>
+      <c r="P14" s="12"/>
+      <c r="Q14" s="12"/>
+      <c r="R14" s="12"/>
+      <c r="S14" s="12"/>
+      <c r="T14" s="12"/>
+      <c r="U14" s="12"/>
+      <c r="V14" s="12"/>
+      <c r="W14" s="12"/>
+      <c r="X14" s="12"/>
+      <c r="Y14" s="12"/>
+      <c r="Z14" s="12"/>
+      <c r="AA14" s="12"/>
+      <c r="AB14" s="12"/>
+      <c r="AC14" s="12"/>
+      <c r="AD14" s="12"/>
+      <c r="AE14" s="12"/>
+      <c r="AF14" s="12"/>
+      <c r="AG14" s="14"/>
+      <c r="AH14" s="14"/>
+      <c r="AI14" s="14"/>
+      <c r="AJ14" s="14"/>
+      <c r="AK14" s="14"/>
+      <c r="AL14" s="14"/>
     </row>
     <row r="15" ht="14.25" customHeight="1">
       <c r="A15" s="10" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>124</v>
-      </c>
-      <c r="C15" s="11"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="11"/>
-      <c r="G15" s="11"/>
-      <c r="H15" s="11"/>
-      <c r="I15" s="11"/>
-      <c r="J15" s="11"/>
-      <c r="K15" s="11"/>
-      <c r="L15" s="11"/>
-      <c r="M15" s="11"/>
-      <c r="N15" s="11" t="s">
-        <v>125</v>
-      </c>
-      <c r="O15" s="11"/>
-      <c r="P15" s="11"/>
-      <c r="Q15" s="11"/>
-      <c r="R15" s="11"/>
-      <c r="S15" s="11"/>
-      <c r="T15" s="11"/>
-      <c r="U15" s="11"/>
-      <c r="V15" s="11"/>
-      <c r="W15" s="11"/>
-      <c r="X15" s="11"/>
-      <c r="Y15" s="11"/>
-      <c r="Z15" s="11"/>
-      <c r="AA15" s="11"/>
-      <c r="AB15" s="11"/>
-      <c r="AC15" s="11"/>
-      <c r="AD15" s="11"/>
-      <c r="AE15" s="11"/>
-      <c r="AF15" s="11"/>
-      <c r="AG15" s="18"/>
-      <c r="AH15" s="18"/>
-      <c r="AI15" s="18"/>
-      <c r="AJ15" s="18"/>
-      <c r="AK15" s="18"/>
-      <c r="AL15" s="18"/>
+        <v>131</v>
+      </c>
+      <c r="C15" s="12"/>
+      <c r="D15" s="12"/>
+      <c r="E15" s="12"/>
+      <c r="F15" s="12"/>
+      <c r="G15" s="12"/>
+      <c r="H15" s="12"/>
+      <c r="I15" s="12"/>
+      <c r="J15" s="12"/>
+      <c r="K15" s="12"/>
+      <c r="L15" s="12"/>
+      <c r="M15" s="12"/>
+      <c r="N15" s="12" t="s">
+        <v>134</v>
+      </c>
+      <c r="O15" s="12"/>
+      <c r="P15" s="12"/>
+      <c r="Q15" s="12"/>
+      <c r="R15" s="12"/>
+      <c r="S15" s="12"/>
+      <c r="T15" s="12"/>
+      <c r="U15" s="12"/>
+      <c r="V15" s="12"/>
+      <c r="W15" s="12"/>
+      <c r="X15" s="12"/>
+      <c r="Y15" s="12"/>
+      <c r="Z15" s="12"/>
+      <c r="AA15" s="12"/>
+      <c r="AB15" s="12"/>
+      <c r="AC15" s="12"/>
+      <c r="AD15" s="12"/>
+      <c r="AE15" s="12"/>
+      <c r="AF15" s="12"/>
+      <c r="AG15" s="14"/>
+      <c r="AH15" s="14"/>
+      <c r="AI15" s="14"/>
+      <c r="AJ15" s="14"/>
+      <c r="AK15" s="14"/>
+      <c r="AL15" s="14"/>
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="10" t="s">
-        <v>106</v>
+        <v>88</v>
       </c>
       <c r="B16" s="10"/>
-      <c r="C16" s="11"/>
-      <c r="D16" s="11"/>
-      <c r="E16" s="11"/>
-      <c r="F16" s="11"/>
-      <c r="G16" s="11"/>
-      <c r="H16" s="11"/>
-      <c r="I16" s="11"/>
-      <c r="J16" s="11"/>
-      <c r="K16" s="11"/>
-      <c r="L16" s="11"/>
-      <c r="M16" s="11"/>
-      <c r="N16" s="11"/>
-      <c r="O16" s="11"/>
-      <c r="P16" s="11"/>
-      <c r="Q16" s="11"/>
-      <c r="R16" s="11"/>
-      <c r="S16" s="11"/>
-      <c r="T16" s="11"/>
-      <c r="U16" s="11"/>
-      <c r="V16" s="11"/>
-      <c r="W16" s="11"/>
-      <c r="X16" s="11"/>
-      <c r="Y16" s="11"/>
-      <c r="Z16" s="11"/>
-      <c r="AA16" s="11"/>
-      <c r="AB16" s="11"/>
-      <c r="AC16" s="11"/>
-      <c r="AD16" s="11"/>
-      <c r="AE16" s="11"/>
-      <c r="AF16" s="11"/>
-      <c r="AG16" s="18"/>
-      <c r="AH16" s="18"/>
-      <c r="AI16" s="18"/>
-      <c r="AJ16" s="18"/>
-      <c r="AK16" s="18"/>
-      <c r="AL16" s="18"/>
+      <c r="C16" s="12"/>
+      <c r="D16" s="12"/>
+      <c r="E16" s="12"/>
+      <c r="F16" s="12"/>
+      <c r="G16" s="12"/>
+      <c r="H16" s="12"/>
+      <c r="I16" s="12"/>
+      <c r="J16" s="12"/>
+      <c r="K16" s="12"/>
+      <c r="L16" s="12"/>
+      <c r="M16" s="12"/>
+      <c r="N16" s="12"/>
+      <c r="O16" s="12"/>
+      <c r="P16" s="12"/>
+      <c r="Q16" s="12"/>
+      <c r="R16" s="12"/>
+      <c r="S16" s="12"/>
+      <c r="T16" s="12"/>
+      <c r="U16" s="12"/>
+      <c r="V16" s="12"/>
+      <c r="W16" s="12"/>
+      <c r="X16" s="12"/>
+      <c r="Y16" s="12"/>
+      <c r="Z16" s="12"/>
+      <c r="AA16" s="12"/>
+      <c r="AB16" s="12"/>
+      <c r="AC16" s="12"/>
+      <c r="AD16" s="12"/>
+      <c r="AE16" s="12"/>
+      <c r="AF16" s="12"/>
+      <c r="AG16" s="14"/>
+      <c r="AH16" s="14"/>
+      <c r="AI16" s="14"/>
+      <c r="AJ16" s="14"/>
+      <c r="AK16" s="14"/>
+      <c r="AL16" s="14"/>
     </row>
     <row r="17" ht="14.25" customHeight="1">
       <c r="D17" s="9"/>
-      <c r="E17" s="26"/>
-      <c r="K17" s="27"/>
+      <c r="E17" s="27"/>
+      <c r="K17" s="28"/>
       <c r="L17" s="9"/>
-      <c r="M17" s="26"/>
+      <c r="M17" s="27"/>
       <c r="Q17" s="9"/>
-      <c r="R17" s="26"/>
+      <c r="R17" s="27"/>
     </row>
     <row r="18" ht="14.25" customHeight="1">
-      <c r="A18" s="28" t="s">
+      <c r="A18" s="29" t="s">
         <v>33</v>
       </c>
-      <c r="B18" s="28" t="s">
-        <v>126</v>
+      <c r="B18" s="29" t="s">
+        <v>137</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="D18" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="E18" s="29" t="s">
-        <v>42</v>
+        <v>41</v>
+      </c>
+      <c r="D18" s="30" t="s">
+        <v>41</v>
+      </c>
+      <c r="E18" s="30" t="s">
+        <v>41</v>
       </c>
       <c r="F18" s="9"/>
       <c r="G18" s="9"/>
@@ -2042,28 +2114,28 @@
       <c r="AD18" s="9"/>
       <c r="AE18" s="9"/>
       <c r="AF18" s="9"/>
-      <c r="AG18" s="26"/>
-      <c r="AH18" s="26"/>
-      <c r="AI18" s="26"/>
-      <c r="AJ18" s="26"/>
-      <c r="AK18" s="26"/>
-      <c r="AL18" s="26"/>
+      <c r="AG18" s="27"/>
+      <c r="AH18" s="27"/>
+      <c r="AI18" s="27"/>
+      <c r="AJ18" s="27"/>
+      <c r="AK18" s="27"/>
+      <c r="AL18" s="27"/>
     </row>
     <row r="19" ht="14.25" customHeight="1">
-      <c r="A19" s="28" t="s">
-        <v>92</v>
-      </c>
-      <c r="B19" s="28" t="s">
-        <v>127</v>
+      <c r="A19" s="29" t="s">
+        <v>87</v>
+      </c>
+      <c r="B19" s="29" t="s">
+        <v>138</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>128</v>
-      </c>
-      <c r="D19" s="29" t="s">
-        <v>129</v>
-      </c>
-      <c r="E19" s="29" t="s">
-        <v>130</v>
+        <v>139</v>
+      </c>
+      <c r="D19" s="30" t="s">
+        <v>140</v>
+      </c>
+      <c r="E19" s="30" t="s">
+        <v>141</v>
       </c>
       <c r="F19" s="9"/>
       <c r="G19" s="9"/>
@@ -2079,7 +2151,7 @@
       <c r="Q19" s="9"/>
       <c r="R19" s="9"/>
       <c r="S19" s="9" t="s">
-        <v>131</v>
+        <v>142</v>
       </c>
       <c r="T19" s="9"/>
       <c r="U19" s="9"/>
@@ -2094,28 +2166,28 @@
       <c r="AD19" s="9"/>
       <c r="AE19" s="9"/>
       <c r="AF19" s="9"/>
-      <c r="AG19" s="26"/>
-      <c r="AH19" s="26"/>
-      <c r="AI19" s="26"/>
-      <c r="AJ19" s="26"/>
-      <c r="AK19" s="26"/>
-      <c r="AL19" s="26"/>
+      <c r="AG19" s="27"/>
+      <c r="AH19" s="27"/>
+      <c r="AI19" s="27"/>
+      <c r="AJ19" s="27"/>
+      <c r="AK19" s="27"/>
+      <c r="AL19" s="27"/>
     </row>
     <row r="20" ht="14.25" customHeight="1">
-      <c r="A20" s="28" t="s">
-        <v>92</v>
-      </c>
-      <c r="B20" s="28" t="s">
+      <c r="A20" s="29" t="s">
+        <v>87</v>
+      </c>
+      <c r="B20" s="29" t="s">
         <v>0</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>132</v>
-      </c>
-      <c r="D20" s="29" t="s">
-        <v>133</v>
-      </c>
-      <c r="E20" s="29" t="s">
-        <v>134</v>
+        <v>143</v>
+      </c>
+      <c r="D20" s="30" t="s">
+        <v>144</v>
+      </c>
+      <c r="E20" s="30" t="s">
+        <v>145</v>
       </c>
       <c r="F20" s="9"/>
       <c r="G20" s="9"/>
@@ -2131,7 +2203,7 @@
       <c r="Q20" s="9"/>
       <c r="R20" s="9"/>
       <c r="S20" s="9" t="s">
-        <v>126</v>
+        <v>137</v>
       </c>
       <c r="T20" s="9"/>
       <c r="U20" s="9"/>
@@ -2146,31 +2218,31 @@
       <c r="AD20" s="9"/>
       <c r="AE20" s="9"/>
       <c r="AF20" s="9"/>
-      <c r="AG20" s="26"/>
-      <c r="AH20" s="26"/>
-      <c r="AI20" s="26"/>
-      <c r="AJ20" s="26"/>
-      <c r="AK20" s="26"/>
-      <c r="AL20" s="26"/>
+      <c r="AG20" s="27"/>
+      <c r="AH20" s="27"/>
+      <c r="AI20" s="27"/>
+      <c r="AJ20" s="27"/>
+      <c r="AK20" s="27"/>
+      <c r="AL20" s="27"/>
     </row>
     <row r="21" ht="14.25" customHeight="1">
-      <c r="A21" s="28" t="s">
-        <v>69</v>
-      </c>
-      <c r="B21" s="28" t="s">
-        <v>1</v>
+      <c r="A21" s="29" t="s">
+        <v>66</v>
+      </c>
+      <c r="B21" s="29" t="s">
+        <v>3</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>135</v>
-      </c>
-      <c r="D21" s="29" t="s">
-        <v>85</v>
-      </c>
-      <c r="E21" s="29" t="s">
-        <v>136</v>
+        <v>146</v>
+      </c>
+      <c r="D21" s="30" t="s">
+        <v>83</v>
+      </c>
+      <c r="E21" s="30" t="s">
+        <v>147</v>
       </c>
       <c r="F21" s="9" t="s">
-        <v>137</v>
+        <v>148</v>
       </c>
       <c r="G21" s="9"/>
       <c r="H21" s="9"/>
@@ -2198,57 +2270,57 @@
       <c r="AD21" s="9"/>
       <c r="AE21" s="9"/>
       <c r="AF21" s="9"/>
-      <c r="AG21" s="26"/>
-      <c r="AH21" s="26"/>
-      <c r="AI21" s="26"/>
-      <c r="AJ21" s="26"/>
-      <c r="AK21" s="26"/>
-      <c r="AL21" s="26"/>
+      <c r="AG21" s="27"/>
+      <c r="AH21" s="27"/>
+      <c r="AI21" s="27"/>
+      <c r="AJ21" s="27"/>
+      <c r="AK21" s="27"/>
+      <c r="AL21" s="27"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
-      <c r="A22" s="28" t="s">
-        <v>69</v>
-      </c>
-      <c r="B22" s="28" t="s">
-        <v>138</v>
+      <c r="A22" s="29" t="s">
+        <v>66</v>
+      </c>
+      <c r="B22" s="29" t="s">
+        <v>149</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>139</v>
-      </c>
-      <c r="D22" s="29" t="s">
-        <v>140</v>
-      </c>
-      <c r="E22" s="29" t="s">
-        <v>141</v>
+        <v>150</v>
+      </c>
+      <c r="D22" s="30" t="s">
+        <v>151</v>
+      </c>
+      <c r="E22" s="30" t="s">
+        <v>152</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>142</v>
+        <v>153</v>
       </c>
       <c r="G22" s="9"/>
       <c r="H22" s="9"/>
       <c r="I22" s="9"/>
       <c r="J22" s="9" t="s">
-        <v>143</v>
+        <v>154</v>
       </c>
       <c r="K22" s="9" t="s">
-        <v>144</v>
-      </c>
-      <c r="L22" s="29" t="s">
-        <v>145</v>
-      </c>
-      <c r="M22" s="29" t="s">
-        <v>146</v>
+        <v>155</v>
+      </c>
+      <c r="L22" s="30" t="s">
+        <v>156</v>
+      </c>
+      <c r="M22" s="30" t="s">
+        <v>157</v>
       </c>
       <c r="N22" s="9"/>
       <c r="O22" s="9"/>
-      <c r="P22" s="30" t="s">
-        <v>147</v>
-      </c>
-      <c r="Q22" s="29" t="s">
-        <v>148</v>
-      </c>
-      <c r="R22" s="29" t="s">
-        <v>149</v>
+      <c r="P22" s="31" t="s">
+        <v>158</v>
+      </c>
+      <c r="Q22" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="R22" s="30" t="s">
+        <v>160</v>
       </c>
       <c r="S22" s="9"/>
       <c r="T22" s="9"/>
@@ -2264,25 +2336,25 @@
       <c r="AD22" s="9"/>
       <c r="AE22" s="9"/>
       <c r="AF22" s="9"/>
-      <c r="AG22" s="26"/>
-      <c r="AH22" s="26"/>
-      <c r="AI22" s="26"/>
-      <c r="AJ22" s="26"/>
-      <c r="AK22" s="26"/>
-      <c r="AL22" s="26"/>
+      <c r="AG22" s="27"/>
+      <c r="AH22" s="27"/>
+      <c r="AI22" s="27"/>
+      <c r="AJ22" s="27"/>
+      <c r="AK22" s="27"/>
+      <c r="AL22" s="27"/>
     </row>
     <row r="23" ht="14.25" customHeight="1">
-      <c r="A23" s="28" t="s">
-        <v>123</v>
-      </c>
-      <c r="B23" s="28" t="s">
-        <v>150</v>
-      </c>
-      <c r="C23" s="31"/>
-      <c r="D23" s="31"/>
-      <c r="E23" s="31"/>
+      <c r="A23" s="29" t="s">
+        <v>130</v>
+      </c>
+      <c r="B23" s="29" t="s">
+        <v>161</v>
+      </c>
+      <c r="C23" s="32"/>
+      <c r="D23" s="32"/>
+      <c r="E23" s="32"/>
       <c r="F23" s="9" t="s">
-        <v>137</v>
+        <v>148</v>
       </c>
       <c r="G23" s="9"/>
       <c r="H23" s="9"/>
@@ -2292,7 +2364,7 @@
       <c r="L23" s="9"/>
       <c r="M23" s="9"/>
       <c r="N23" s="9" t="s">
-        <v>151</v>
+        <v>162</v>
       </c>
       <c r="O23" s="9"/>
       <c r="P23" s="9"/>
@@ -2312,21 +2384,21 @@
       <c r="AD23" s="9"/>
       <c r="AE23" s="9"/>
       <c r="AF23" s="9"/>
-      <c r="AG23" s="26"/>
-      <c r="AH23" s="26"/>
-      <c r="AI23" s="26"/>
-      <c r="AJ23" s="26"/>
-      <c r="AK23" s="26"/>
-      <c r="AL23" s="26"/>
+      <c r="AG23" s="27"/>
+      <c r="AH23" s="27"/>
+      <c r="AI23" s="27"/>
+      <c r="AJ23" s="27"/>
+      <c r="AK23" s="27"/>
+      <c r="AL23" s="27"/>
     </row>
     <row r="24" ht="14.25" customHeight="1">
-      <c r="A24" s="28" t="s">
-        <v>123</v>
-      </c>
-      <c r="B24" s="28" t="s">
-        <v>152</v>
-      </c>
-      <c r="C24" s="31"/>
+      <c r="A24" s="29" t="s">
+        <v>130</v>
+      </c>
+      <c r="B24" s="29" t="s">
+        <v>163</v>
+      </c>
+      <c r="C24" s="32"/>
       <c r="D24" s="9"/>
       <c r="E24" s="9"/>
       <c r="F24" s="9"/>
@@ -2338,7 +2410,7 @@
       <c r="L24" s="9"/>
       <c r="M24" s="9"/>
       <c r="N24" s="9" t="s">
-        <v>153</v>
+        <v>164</v>
       </c>
       <c r="O24" s="9"/>
       <c r="P24" s="9"/>
@@ -2358,28 +2430,28 @@
       <c r="AD24" s="9"/>
       <c r="AE24" s="9"/>
       <c r="AF24" s="9"/>
-      <c r="AG24" s="26"/>
-      <c r="AH24" s="26"/>
-      <c r="AI24" s="26"/>
-      <c r="AJ24" s="26"/>
-      <c r="AK24" s="26"/>
-      <c r="AL24" s="26"/>
+      <c r="AG24" s="27"/>
+      <c r="AH24" s="27"/>
+      <c r="AI24" s="27"/>
+      <c r="AJ24" s="27"/>
+      <c r="AK24" s="27"/>
+      <c r="AL24" s="27"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
-      <c r="A25" s="28" t="s">
+      <c r="A25" s="29" t="s">
         <v>33</v>
       </c>
-      <c r="B25" s="28" t="s">
-        <v>154</v>
+      <c r="B25" s="29" t="s">
+        <v>165</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="D25" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="E25" s="29" t="s">
-        <v>42</v>
+        <v>41</v>
+      </c>
+      <c r="D25" s="30" t="s">
+        <v>41</v>
+      </c>
+      <c r="E25" s="30" t="s">
+        <v>41</v>
       </c>
       <c r="F25" s="9"/>
       <c r="G25" s="9"/>
@@ -2408,59 +2480,59 @@
       <c r="AD25" s="9"/>
       <c r="AE25" s="9"/>
       <c r="AF25" s="9"/>
-      <c r="AG25" s="26"/>
-      <c r="AH25" s="26"/>
-      <c r="AI25" s="26"/>
-      <c r="AJ25" s="26"/>
-      <c r="AK25" s="26"/>
-      <c r="AL25" s="26"/>
+      <c r="AG25" s="27"/>
+      <c r="AH25" s="27"/>
+      <c r="AI25" s="27"/>
+      <c r="AJ25" s="27"/>
+      <c r="AK25" s="27"/>
+      <c r="AL25" s="27"/>
     </row>
     <row r="26" ht="14.25" customHeight="1">
-      <c r="A26" s="28" t="s">
-        <v>155</v>
-      </c>
-      <c r="B26" s="28" t="s">
-        <v>156</v>
+      <c r="A26" s="29" t="s">
+        <v>166</v>
+      </c>
+      <c r="B26" s="29" t="s">
+        <v>167</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>157</v>
-      </c>
-      <c r="D26" s="29" t="s">
-        <v>158</v>
-      </c>
-      <c r="E26" s="29" t="s">
-        <v>159</v>
+        <v>168</v>
+      </c>
+      <c r="D26" s="30" t="s">
+        <v>169</v>
+      </c>
+      <c r="E26" s="30" t="s">
+        <v>170</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>137</v>
+        <v>148</v>
       </c>
       <c r="G26" s="9" t="s">
-        <v>160</v>
+        <v>171</v>
       </c>
       <c r="H26" s="9"/>
       <c r="I26" s="9"/>
       <c r="J26" s="9" t="s">
-        <v>161</v>
+        <v>172</v>
       </c>
       <c r="K26" s="9" t="s">
-        <v>162</v>
-      </c>
-      <c r="L26" s="29" t="s">
-        <v>163</v>
-      </c>
-      <c r="M26" s="29" t="s">
-        <v>164</v>
+        <v>173</v>
+      </c>
+      <c r="L26" s="30" t="s">
+        <v>174</v>
+      </c>
+      <c r="M26" s="30" t="s">
+        <v>175</v>
       </c>
       <c r="N26" s="9"/>
       <c r="O26" s="9"/>
       <c r="P26" s="9" t="s">
-        <v>165</v>
-      </c>
-      <c r="Q26" s="29" t="s">
-        <v>166</v>
-      </c>
-      <c r="R26" s="29" t="s">
-        <v>167</v>
+        <v>176</v>
+      </c>
+      <c r="Q26" s="30" t="s">
+        <v>177</v>
+      </c>
+      <c r="R26" s="30" t="s">
+        <v>178</v>
       </c>
       <c r="S26" s="9"/>
       <c r="T26" s="9"/>
@@ -2476,32 +2548,32 @@
       <c r="AD26" s="9"/>
       <c r="AE26" s="9"/>
       <c r="AF26" s="9"/>
-      <c r="AG26" s="26"/>
-      <c r="AH26" s="26"/>
-      <c r="AI26" s="26"/>
-      <c r="AJ26" s="26"/>
-      <c r="AK26" s="26"/>
-      <c r="AL26" s="26"/>
+      <c r="AG26" s="27"/>
+      <c r="AH26" s="27"/>
+      <c r="AI26" s="27"/>
+      <c r="AJ26" s="27"/>
+      <c r="AK26" s="27"/>
+      <c r="AL26" s="27"/>
     </row>
     <row r="27" ht="14.25" customHeight="1">
-      <c r="A27" s="28" t="s">
-        <v>168</v>
-      </c>
-      <c r="B27" s="28" t="s">
-        <v>169</v>
+      <c r="A27" s="29" t="s">
+        <v>179</v>
+      </c>
+      <c r="B27" s="29" t="s">
+        <v>180</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>170</v>
-      </c>
-      <c r="D27" s="29" t="s">
-        <v>171</v>
-      </c>
-      <c r="E27" s="29" t="s">
-        <v>172</v>
+        <v>181</v>
+      </c>
+      <c r="D27" s="30" t="s">
+        <v>182</v>
+      </c>
+      <c r="E27" s="30" t="s">
+        <v>183</v>
       </c>
       <c r="F27" s="9"/>
       <c r="G27" s="9" t="s">
-        <v>173</v>
+        <v>184</v>
       </c>
       <c r="H27" s="9"/>
       <c r="I27" s="9"/>
@@ -2528,48 +2600,48 @@
       <c r="AD27" s="9"/>
       <c r="AE27" s="9"/>
       <c r="AF27" s="9"/>
-      <c r="AG27" s="26"/>
-      <c r="AH27" s="26"/>
-      <c r="AI27" s="26"/>
-      <c r="AJ27" s="26"/>
-      <c r="AK27" s="26"/>
-      <c r="AL27" s="26"/>
+      <c r="AG27" s="27"/>
+      <c r="AH27" s="27"/>
+      <c r="AI27" s="27"/>
+      <c r="AJ27" s="27"/>
+      <c r="AK27" s="27"/>
+      <c r="AL27" s="27"/>
     </row>
     <row r="28" ht="14.25" customHeight="1">
-      <c r="A28" s="28" t="s">
-        <v>174</v>
-      </c>
-      <c r="B28" s="28" t="s">
-        <v>175</v>
+      <c r="A28" s="29" t="s">
+        <v>185</v>
+      </c>
+      <c r="B28" s="29" t="s">
+        <v>186</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>176</v>
-      </c>
-      <c r="D28" s="29" t="s">
-        <v>177</v>
-      </c>
-      <c r="E28" s="29" t="s">
-        <v>178</v>
+        <v>187</v>
+      </c>
+      <c r="D28" s="30" t="s">
+        <v>188</v>
+      </c>
+      <c r="E28" s="30" t="s">
+        <v>189</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>137</v>
+        <v>148</v>
       </c>
       <c r="G28" s="9" t="s">
-        <v>173</v>
+        <v>184</v>
       </c>
       <c r="H28" s="9"/>
       <c r="I28" s="9"/>
       <c r="J28" s="9" t="s">
-        <v>179</v>
+        <v>190</v>
       </c>
       <c r="K28" s="9" t="s">
-        <v>180</v>
-      </c>
-      <c r="L28" s="29" t="s">
-        <v>181</v>
-      </c>
-      <c r="M28" s="29" t="s">
-        <v>182</v>
+        <v>191</v>
+      </c>
+      <c r="L28" s="30" t="s">
+        <v>192</v>
+      </c>
+      <c r="M28" s="30" t="s">
+        <v>193</v>
       </c>
       <c r="N28" s="9"/>
       <c r="O28" s="9"/>
@@ -2590,46 +2662,46 @@
       <c r="AD28" s="9"/>
       <c r="AE28" s="9"/>
       <c r="AF28" s="9"/>
-      <c r="AG28" s="26"/>
-      <c r="AH28" s="26"/>
-      <c r="AI28" s="26"/>
-      <c r="AJ28" s="26"/>
-      <c r="AK28" s="26"/>
-      <c r="AL28" s="26"/>
+      <c r="AG28" s="27"/>
+      <c r="AH28" s="27"/>
+      <c r="AI28" s="27"/>
+      <c r="AJ28" s="27"/>
+      <c r="AK28" s="27"/>
+      <c r="AL28" s="27"/>
     </row>
     <row r="29" ht="14.25" customHeight="1">
-      <c r="A29" s="28" t="s">
-        <v>174</v>
-      </c>
-      <c r="B29" s="28" t="s">
-        <v>183</v>
+      <c r="A29" s="29" t="s">
+        <v>185</v>
+      </c>
+      <c r="B29" s="29" t="s">
+        <v>194</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>184</v>
-      </c>
-      <c r="D29" s="29" t="s">
-        <v>185</v>
-      </c>
-      <c r="E29" s="29" t="s">
-        <v>186</v>
+        <v>195</v>
+      </c>
+      <c r="D29" s="30" t="s">
+        <v>196</v>
+      </c>
+      <c r="E29" s="30" t="s">
+        <v>197</v>
       </c>
       <c r="F29" s="9"/>
       <c r="G29" s="9" t="s">
-        <v>173</v>
+        <v>184</v>
       </c>
       <c r="H29" s="9"/>
       <c r="I29" s="9"/>
       <c r="J29" s="9" t="s">
-        <v>187</v>
+        <v>198</v>
       </c>
       <c r="K29" s="9" t="s">
-        <v>188</v>
-      </c>
-      <c r="L29" s="29" t="s">
-        <v>189</v>
-      </c>
-      <c r="M29" s="29" t="s">
-        <v>190</v>
+        <v>199</v>
+      </c>
+      <c r="L29" s="30" t="s">
+        <v>200</v>
+      </c>
+      <c r="M29" s="30" t="s">
+        <v>201</v>
       </c>
       <c r="N29" s="9"/>
       <c r="O29" s="9"/>
@@ -2650,29 +2722,29 @@
       <c r="AD29" s="9"/>
       <c r="AE29" s="9"/>
       <c r="AF29" s="9"/>
-      <c r="AG29" s="26"/>
-      <c r="AH29" s="26"/>
-      <c r="AI29" s="26"/>
-      <c r="AJ29" s="26"/>
-      <c r="AK29" s="26"/>
-      <c r="AL29" s="26"/>
+      <c r="AG29" s="27"/>
+      <c r="AH29" s="27"/>
+      <c r="AI29" s="27"/>
+      <c r="AJ29" s="27"/>
+      <c r="AK29" s="27"/>
+      <c r="AL29" s="27"/>
     </row>
     <row r="30" ht="14.25" customHeight="1">
-      <c r="A30" s="28" t="s">
-        <v>191</v>
-      </c>
-      <c r="B30" s="28" t="s">
-        <v>192</v>
+      <c r="A30" s="29" t="s">
+        <v>202</v>
+      </c>
+      <c r="B30" s="29" t="s">
+        <v>203</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>193</v>
+        <v>204</v>
       </c>
       <c r="D30" s="9"/>
       <c r="E30" s="9"/>
       <c r="F30" s="9"/>
       <c r="G30" s="9"/>
       <c r="H30" s="9" t="s">
-        <v>194</v>
+        <v>205</v>
       </c>
       <c r="I30" s="9"/>
       <c r="J30" s="9"/>
@@ -2698,21 +2770,21 @@
       <c r="AD30" s="9"/>
       <c r="AE30" s="9"/>
       <c r="AF30" s="9"/>
-      <c r="AG30" s="26"/>
-      <c r="AH30" s="26"/>
-      <c r="AI30" s="26"/>
-      <c r="AJ30" s="26"/>
-      <c r="AK30" s="26"/>
-      <c r="AL30" s="26"/>
+      <c r="AG30" s="27"/>
+      <c r="AH30" s="27"/>
+      <c r="AI30" s="27"/>
+      <c r="AJ30" s="27"/>
+      <c r="AK30" s="27"/>
+      <c r="AL30" s="27"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
-      <c r="A31" s="28" t="s">
-        <v>123</v>
-      </c>
-      <c r="B31" s="28" t="s">
-        <v>195</v>
-      </c>
-      <c r="C31" s="31"/>
+      <c r="A31" s="29" t="s">
+        <v>130</v>
+      </c>
+      <c r="B31" s="29" t="s">
+        <v>206</v>
+      </c>
+      <c r="C31" s="32"/>
       <c r="D31" s="9"/>
       <c r="E31" s="9"/>
       <c r="F31" s="9"/>
@@ -2723,8 +2795,8 @@
       <c r="K31" s="9"/>
       <c r="L31" s="9"/>
       <c r="M31" s="9"/>
-      <c r="N31" s="31" t="s">
-        <v>196</v>
+      <c r="N31" s="32" t="s">
+        <v>207</v>
       </c>
       <c r="O31" s="9"/>
       <c r="P31" s="9"/>
@@ -2744,19 +2816,19 @@
       <c r="AD31" s="9"/>
       <c r="AE31" s="9"/>
       <c r="AF31" s="9"/>
-      <c r="AG31" s="26"/>
-      <c r="AH31" s="26"/>
-      <c r="AI31" s="26"/>
-      <c r="AJ31" s="26"/>
-      <c r="AK31" s="26"/>
-      <c r="AL31" s="26"/>
+      <c r="AG31" s="27"/>
+      <c r="AH31" s="27"/>
+      <c r="AI31" s="27"/>
+      <c r="AJ31" s="27"/>
+      <c r="AK31" s="27"/>
+      <c r="AL31" s="27"/>
     </row>
     <row r="32" ht="14.25" customHeight="1">
-      <c r="A32" s="28" t="s">
-        <v>123</v>
-      </c>
-      <c r="B32" s="28" t="s">
-        <v>197</v>
+      <c r="A32" s="29" t="s">
+        <v>130</v>
+      </c>
+      <c r="B32" s="29" t="s">
+        <v>208</v>
       </c>
       <c r="C32" s="9"/>
       <c r="D32" s="9"/>
@@ -2769,8 +2841,8 @@
       <c r="K32" s="9"/>
       <c r="L32" s="9"/>
       <c r="M32" s="9"/>
-      <c r="N32" s="32" t="s">
-        <v>198</v>
+      <c r="N32" s="33" t="s">
+        <v>209</v>
       </c>
       <c r="O32" s="9"/>
       <c r="P32" s="9"/>
@@ -2790,21 +2862,21 @@
       <c r="AD32" s="9"/>
       <c r="AE32" s="9"/>
       <c r="AF32" s="9"/>
-      <c r="AG32" s="26"/>
-      <c r="AH32" s="26"/>
-      <c r="AI32" s="26"/>
-      <c r="AJ32" s="26"/>
-      <c r="AK32" s="26"/>
-      <c r="AL32" s="26"/>
+      <c r="AG32" s="27"/>
+      <c r="AH32" s="27"/>
+      <c r="AI32" s="27"/>
+      <c r="AJ32" s="27"/>
+      <c r="AK32" s="27"/>
+      <c r="AL32" s="27"/>
     </row>
     <row r="33" ht="14.25" customHeight="1">
-      <c r="A33" s="28" t="s">
-        <v>123</v>
-      </c>
-      <c r="B33" s="28" t="s">
-        <v>199</v>
-      </c>
-      <c r="C33" s="31"/>
+      <c r="A33" s="29" t="s">
+        <v>130</v>
+      </c>
+      <c r="B33" s="29" t="s">
+        <v>210</v>
+      </c>
+      <c r="C33" s="32"/>
       <c r="D33" s="9"/>
       <c r="E33" s="9"/>
       <c r="F33" s="9"/>
@@ -2816,7 +2888,7 @@
       <c r="L33" s="9"/>
       <c r="M33" s="9"/>
       <c r="N33" s="9" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
       <c r="O33" s="9"/>
       <c r="P33" s="9"/>
@@ -2836,28 +2908,28 @@
       <c r="AD33" s="9"/>
       <c r="AE33" s="9"/>
       <c r="AF33" s="9"/>
-      <c r="AG33" s="26"/>
-      <c r="AH33" s="26"/>
-      <c r="AI33" s="26"/>
-      <c r="AJ33" s="26"/>
-      <c r="AK33" s="26"/>
-      <c r="AL33" s="26"/>
+      <c r="AG33" s="27"/>
+      <c r="AH33" s="27"/>
+      <c r="AI33" s="27"/>
+      <c r="AJ33" s="27"/>
+      <c r="AK33" s="27"/>
+      <c r="AL33" s="27"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
-      <c r="A34" s="28" t="s">
-        <v>168</v>
-      </c>
-      <c r="B34" s="28" t="s">
-        <v>201</v>
-      </c>
-      <c r="C34" s="33" t="s">
-        <v>202</v>
+      <c r="A34" s="29" t="s">
+        <v>179</v>
+      </c>
+      <c r="B34" s="29" t="s">
+        <v>212</v>
+      </c>
+      <c r="C34" s="34" t="s">
+        <v>213</v>
       </c>
       <c r="D34" s="9"/>
       <c r="E34" s="9"/>
       <c r="F34" s="9"/>
       <c r="G34" s="9" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="H34" s="9"/>
       <c r="I34" s="9"/>
@@ -2884,18 +2956,18 @@
       <c r="AD34" s="9"/>
       <c r="AE34" s="9"/>
       <c r="AF34" s="9"/>
-      <c r="AG34" s="26"/>
-      <c r="AH34" s="26"/>
-      <c r="AI34" s="26"/>
-      <c r="AJ34" s="26"/>
-      <c r="AK34" s="26"/>
-      <c r="AL34" s="26"/>
+      <c r="AG34" s="27"/>
+      <c r="AH34" s="27"/>
+      <c r="AI34" s="27"/>
+      <c r="AJ34" s="27"/>
+      <c r="AK34" s="27"/>
+      <c r="AL34" s="27"/>
     </row>
     <row r="35" ht="14.25" customHeight="1">
-      <c r="A35" s="28" t="s">
-        <v>106</v>
-      </c>
-      <c r="B35" s="28"/>
+      <c r="A35" s="29" t="s">
+        <v>88</v>
+      </c>
+      <c r="B35" s="29"/>
       <c r="C35" s="9"/>
       <c r="D35" s="9"/>
       <c r="E35" s="9"/>
@@ -2926,38 +2998,38 @@
       <c r="AD35" s="9"/>
       <c r="AE35" s="9"/>
       <c r="AF35" s="9"/>
-      <c r="AG35" s="26"/>
-      <c r="AH35" s="26"/>
-      <c r="AI35" s="26"/>
-      <c r="AJ35" s="26"/>
-      <c r="AK35" s="26"/>
-      <c r="AL35" s="26"/>
+      <c r="AG35" s="27"/>
+      <c r="AH35" s="27"/>
+      <c r="AI35" s="27"/>
+      <c r="AJ35" s="27"/>
+      <c r="AK35" s="27"/>
+      <c r="AL35" s="27"/>
     </row>
     <row r="36" ht="14.25" customHeight="1">
-      <c r="A36" s="28" t="s">
-        <v>203</v>
-      </c>
-      <c r="B36" s="28" t="s">
-        <v>204</v>
+      <c r="A36" s="29" t="s">
+        <v>214</v>
+      </c>
+      <c r="B36" s="29" t="s">
+        <v>215</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>205</v>
-      </c>
-      <c r="D36" s="29" t="s">
-        <v>206</v>
-      </c>
-      <c r="E36" s="29" t="s">
-        <v>207</v>
+        <v>216</v>
+      </c>
+      <c r="D36" s="30" t="s">
+        <v>217</v>
+      </c>
+      <c r="E36" s="30" t="s">
+        <v>218</v>
       </c>
       <c r="F36" s="9" t="s">
-        <v>137</v>
+        <v>148</v>
       </c>
       <c r="G36" s="9"/>
       <c r="H36" s="9" t="s">
-        <v>194</v>
+        <v>205</v>
       </c>
       <c r="I36" s="9"/>
-      <c r="J36" s="29"/>
+      <c r="J36" s="30"/>
       <c r="K36" s="9"/>
       <c r="L36" s="9"/>
       <c r="M36" s="9"/>
@@ -2980,44 +3052,44 @@
       <c r="AD36" s="9"/>
       <c r="AE36" s="9"/>
       <c r="AF36" s="9"/>
-      <c r="AG36" s="26"/>
-      <c r="AH36" s="26"/>
-      <c r="AI36" s="26"/>
-      <c r="AJ36" s="26"/>
-      <c r="AK36" s="26"/>
-      <c r="AL36" s="26"/>
+      <c r="AG36" s="27"/>
+      <c r="AH36" s="27"/>
+      <c r="AI36" s="27"/>
+      <c r="AJ36" s="27"/>
+      <c r="AK36" s="27"/>
+      <c r="AL36" s="27"/>
     </row>
     <row r="37" ht="14.25" customHeight="1">
-      <c r="A37" s="28" t="s">
-        <v>208</v>
-      </c>
-      <c r="B37" s="28" t="s">
-        <v>209</v>
+      <c r="A37" s="29" t="s">
+        <v>219</v>
+      </c>
+      <c r="B37" s="29" t="s">
+        <v>220</v>
       </c>
       <c r="C37" s="9" t="s">
-        <v>210</v>
-      </c>
-      <c r="D37" s="29" t="s">
-        <v>211</v>
-      </c>
-      <c r="E37" s="29" t="s">
-        <v>212</v>
+        <v>221</v>
+      </c>
+      <c r="D37" s="30" t="s">
+        <v>222</v>
+      </c>
+      <c r="E37" s="30" t="s">
+        <v>223</v>
       </c>
       <c r="F37" s="9"/>
       <c r="G37" s="9"/>
       <c r="H37" s="9"/>
       <c r="I37" s="9"/>
       <c r="J37" s="9" t="s">
-        <v>213</v>
+        <v>224</v>
       </c>
       <c r="K37" s="9" t="s">
-        <v>214</v>
-      </c>
-      <c r="L37" s="29" t="s">
-        <v>215</v>
-      </c>
-      <c r="M37" s="29" t="s">
-        <v>216</v>
+        <v>225</v>
+      </c>
+      <c r="L37" s="30" t="s">
+        <v>226</v>
+      </c>
+      <c r="M37" s="30" t="s">
+        <v>227</v>
       </c>
       <c r="N37" s="9"/>
       <c r="O37" s="9"/>
@@ -3038,44 +3110,44 @@
       <c r="AD37" s="9"/>
       <c r="AE37" s="9"/>
       <c r="AF37" s="9"/>
-      <c r="AG37" s="26"/>
-      <c r="AH37" s="26"/>
-      <c r="AI37" s="26"/>
-      <c r="AJ37" s="26"/>
-      <c r="AK37" s="26"/>
-      <c r="AL37" s="26"/>
+      <c r="AG37" s="27"/>
+      <c r="AH37" s="27"/>
+      <c r="AI37" s="27"/>
+      <c r="AJ37" s="27"/>
+      <c r="AK37" s="27"/>
+      <c r="AL37" s="27"/>
     </row>
     <row r="38" ht="14.25" customHeight="1">
-      <c r="A38" s="28" t="s">
-        <v>208</v>
-      </c>
-      <c r="B38" s="28" t="s">
-        <v>217</v>
+      <c r="A38" s="29" t="s">
+        <v>219</v>
+      </c>
+      <c r="B38" s="29" t="s">
+        <v>228</v>
       </c>
       <c r="C38" s="9" t="s">
-        <v>218</v>
-      </c>
-      <c r="D38" s="29" t="s">
-        <v>219</v>
-      </c>
-      <c r="E38" s="29" t="s">
-        <v>220</v>
+        <v>229</v>
+      </c>
+      <c r="D38" s="30" t="s">
+        <v>230</v>
+      </c>
+      <c r="E38" s="30" t="s">
+        <v>231</v>
       </c>
       <c r="F38" s="9"/>
       <c r="G38" s="9"/>
       <c r="H38" s="9"/>
       <c r="I38" s="9"/>
       <c r="J38" s="9" t="s">
-        <v>213</v>
+        <v>224</v>
       </c>
       <c r="K38" s="9" t="s">
-        <v>214</v>
-      </c>
-      <c r="L38" s="29" t="s">
-        <v>215</v>
-      </c>
-      <c r="M38" s="29" t="s">
-        <v>216</v>
+        <v>225</v>
+      </c>
+      <c r="L38" s="30" t="s">
+        <v>226</v>
+      </c>
+      <c r="M38" s="30" t="s">
+        <v>227</v>
       </c>
       <c r="N38" s="9"/>
       <c r="O38" s="9"/>
@@ -3096,35 +3168,35 @@
       <c r="AD38" s="9"/>
       <c r="AE38" s="9"/>
       <c r="AF38" s="9"/>
-      <c r="AG38" s="26"/>
-      <c r="AH38" s="26"/>
-      <c r="AI38" s="26"/>
-      <c r="AJ38" s="26"/>
-      <c r="AK38" s="26"/>
-      <c r="AL38" s="26"/>
+      <c r="AG38" s="27"/>
+      <c r="AH38" s="27"/>
+      <c r="AI38" s="27"/>
+      <c r="AJ38" s="27"/>
+      <c r="AK38" s="27"/>
+      <c r="AL38" s="27"/>
     </row>
     <row r="39" ht="14.25" customHeight="1">
-      <c r="A39" s="28" t="s">
-        <v>221</v>
-      </c>
-      <c r="B39" s="28" t="s">
-        <v>222</v>
+      <c r="A39" s="29" t="s">
+        <v>232</v>
+      </c>
+      <c r="B39" s="29" t="s">
+        <v>233</v>
       </c>
       <c r="C39" s="9" t="s">
-        <v>223</v>
-      </c>
-      <c r="D39" s="29" t="s">
-        <v>224</v>
-      </c>
-      <c r="E39" s="29" t="s">
-        <v>225</v>
+        <v>234</v>
+      </c>
+      <c r="D39" s="30" t="s">
+        <v>235</v>
+      </c>
+      <c r="E39" s="30" t="s">
+        <v>236</v>
       </c>
       <c r="F39" s="9"/>
       <c r="G39" s="9"/>
       <c r="H39" s="9"/>
       <c r="I39" s="9"/>
-      <c r="J39" s="29" t="s">
-        <v>226</v>
+      <c r="J39" s="30" t="s">
+        <v>237</v>
       </c>
       <c r="K39" s="9"/>
       <c r="L39" s="9"/>
@@ -3132,13 +3204,13 @@
       <c r="N39" s="9"/>
       <c r="O39" s="9"/>
       <c r="P39" s="9" t="s">
-        <v>227</v>
-      </c>
-      <c r="Q39" s="29" t="s">
-        <v>228</v>
-      </c>
-      <c r="R39" s="29" t="s">
-        <v>229</v>
+        <v>238</v>
+      </c>
+      <c r="Q39" s="30" t="s">
+        <v>239</v>
+      </c>
+      <c r="R39" s="30" t="s">
+        <v>240</v>
       </c>
       <c r="S39" s="9"/>
       <c r="T39" s="9"/>
@@ -3154,34 +3226,34 @@
       <c r="AD39" s="9"/>
       <c r="AE39" s="9"/>
       <c r="AF39" s="9"/>
-      <c r="AG39" s="26"/>
-      <c r="AH39" s="26"/>
-      <c r="AI39" s="26"/>
-      <c r="AJ39" s="26"/>
-      <c r="AK39" s="26"/>
-      <c r="AL39" s="26"/>
+      <c r="AG39" s="27"/>
+      <c r="AH39" s="27"/>
+      <c r="AI39" s="27"/>
+      <c r="AJ39" s="27"/>
+      <c r="AK39" s="27"/>
+      <c r="AL39" s="27"/>
     </row>
     <row r="40" ht="14.25" customHeight="1">
-      <c r="A40" s="28" t="s">
-        <v>69</v>
-      </c>
-      <c r="B40" s="28" t="s">
-        <v>230</v>
+      <c r="A40" s="29" t="s">
+        <v>66</v>
+      </c>
+      <c r="B40" s="29" t="s">
+        <v>241</v>
       </c>
       <c r="C40" s="9" t="s">
-        <v>231</v>
-      </c>
-      <c r="D40" s="29" t="s">
-        <v>232</v>
-      </c>
-      <c r="E40" s="29" t="s">
-        <v>233</v>
+        <v>242</v>
+      </c>
+      <c r="D40" s="30" t="s">
+        <v>243</v>
+      </c>
+      <c r="E40" s="30" t="s">
+        <v>244</v>
       </c>
       <c r="F40" s="9" t="s">
-        <v>137</v>
+        <v>148</v>
       </c>
       <c r="G40" s="9" t="s">
-        <v>234</v>
+        <v>245</v>
       </c>
       <c r="H40" s="9"/>
       <c r="I40" s="9"/>
@@ -3208,30 +3280,34 @@
       <c r="AD40" s="9"/>
       <c r="AE40" s="9"/>
       <c r="AF40" s="9"/>
-      <c r="AG40" s="26"/>
-      <c r="AH40" s="26"/>
-      <c r="AI40" s="26"/>
-      <c r="AJ40" s="26"/>
-      <c r="AK40" s="26"/>
-      <c r="AL40" s="26"/>
+      <c r="AG40" s="27"/>
+      <c r="AH40" s="27"/>
+      <c r="AI40" s="27"/>
+      <c r="AJ40" s="27"/>
+      <c r="AK40" s="27"/>
+      <c r="AL40" s="27"/>
     </row>
     <row r="41" ht="14.25" customHeight="1">
-      <c r="A41" s="28" t="s">
-        <v>69</v>
-      </c>
-      <c r="B41" s="28" t="s">
-        <v>235</v>
-      </c>
-      <c r="C41" s="9" t="s">
-        <v>236</v>
-      </c>
-      <c r="D41" s="29" t="s">
-        <v>237</v>
-      </c>
-      <c r="E41" s="29" t="s">
-        <v>238</v>
-      </c>
-      <c r="F41" s="9"/>
+      <c r="A41" s="35" t="s">
+        <v>246</v>
+      </c>
+      <c r="B41" s="35" t="s">
+        <v>120</v>
+      </c>
+      <c r="C41" s="30" t="s">
+        <v>247</v>
+      </c>
+      <c r="D41" s="36" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("GOOGLETRANSLATE(C41,""en"",""fr"")"),"**Sélectionnez tous les diagnostics antérieurs de la personne.**")</f>
+        <v>**Sélectionnez tous les diagnostics antérieurs de la personne.**</v>
+      </c>
+      <c r="E41" s="36" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("GOOGLETRANSLATE(C41,""en"",""ht"")"),"**Chwazi tout sa moun nan te deja dyagnostike avèk yo**")</f>
+        <v>**Chwazi tout sa moun nan te deja dyagnostike avèk yo**</v>
+      </c>
+      <c r="F41" s="30" t="s">
+        <v>148</v>
+      </c>
       <c r="G41" s="9"/>
       <c r="H41" s="9"/>
       <c r="I41" s="9"/>
@@ -3258,40 +3334,36 @@
       <c r="AD41" s="9"/>
       <c r="AE41" s="9"/>
       <c r="AF41" s="9"/>
-      <c r="AG41" s="26"/>
-      <c r="AH41" s="26"/>
-      <c r="AI41" s="26"/>
-      <c r="AJ41" s="26"/>
-      <c r="AK41" s="26"/>
-      <c r="AL41" s="26"/>
+      <c r="AG41" s="27"/>
+      <c r="AH41" s="27"/>
+      <c r="AI41" s="27"/>
+      <c r="AJ41" s="27"/>
+      <c r="AK41" s="27"/>
+      <c r="AL41" s="27"/>
     </row>
     <row r="42" ht="14.25" customHeight="1">
-      <c r="A42" s="28" t="s">
-        <v>69</v>
-      </c>
-      <c r="B42" s="28" t="s">
-        <v>239</v>
-      </c>
-      <c r="C42" s="9" t="s">
-        <v>240</v>
-      </c>
-      <c r="D42" s="29" t="s">
-        <v>240</v>
-      </c>
-      <c r="E42" s="29" t="s">
-        <v>241</v>
-      </c>
-      <c r="F42" s="9"/>
+      <c r="A42" s="35" t="s">
+        <v>130</v>
+      </c>
+      <c r="B42" s="35" t="s">
+        <v>248</v>
+      </c>
+      <c r="C42" s="30" t="s">
+        <v>41</v>
+      </c>
+      <c r="D42" s="36"/>
+      <c r="E42" s="36"/>
+      <c r="F42" s="30"/>
       <c r="G42" s="9"/>
-      <c r="H42" s="9" t="s">
-        <v>242</v>
-      </c>
+      <c r="H42" s="9"/>
       <c r="I42" s="9"/>
       <c r="J42" s="9"/>
       <c r="K42" s="9"/>
       <c r="L42" s="9"/>
       <c r="M42" s="9"/>
-      <c r="N42" s="9"/>
+      <c r="N42" s="30" t="s">
+        <v>249</v>
+      </c>
       <c r="O42" s="9"/>
       <c r="P42" s="9"/>
       <c r="Q42" s="9"/>
@@ -3310,30 +3382,26 @@
       <c r="AD42" s="9"/>
       <c r="AE42" s="9"/>
       <c r="AF42" s="9"/>
-      <c r="AG42" s="26"/>
-      <c r="AH42" s="26"/>
-      <c r="AI42" s="26"/>
-      <c r="AJ42" s="26"/>
-      <c r="AK42" s="26"/>
-      <c r="AL42" s="26"/>
+      <c r="AG42" s="27"/>
+      <c r="AH42" s="27"/>
+      <c r="AI42" s="27"/>
+      <c r="AJ42" s="27"/>
+      <c r="AK42" s="27"/>
+      <c r="AL42" s="27"/>
     </row>
     <row r="43" ht="14.25" customHeight="1">
-      <c r="A43" s="28" t="s">
-        <v>33</v>
-      </c>
-      <c r="B43" s="28" t="s">
-        <v>243</v>
-      </c>
-      <c r="C43" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="D43" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="E43" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="F43" s="9"/>
+      <c r="A43" s="35" t="s">
+        <v>130</v>
+      </c>
+      <c r="B43" s="35" t="s">
+        <v>250</v>
+      </c>
+      <c r="C43" s="30" t="s">
+        <v>41</v>
+      </c>
+      <c r="D43" s="36"/>
+      <c r="E43" s="36"/>
+      <c r="F43" s="30"/>
       <c r="G43" s="9"/>
       <c r="H43" s="9"/>
       <c r="I43" s="9"/>
@@ -3341,7 +3409,9 @@
       <c r="K43" s="9"/>
       <c r="L43" s="9"/>
       <c r="M43" s="9"/>
-      <c r="N43" s="9"/>
+      <c r="N43" s="30" t="s">
+        <v>251</v>
+      </c>
       <c r="O43" s="9"/>
       <c r="P43" s="9"/>
       <c r="Q43" s="9"/>
@@ -3360,24 +3430,26 @@
       <c r="AD43" s="9"/>
       <c r="AE43" s="9"/>
       <c r="AF43" s="9"/>
-      <c r="AG43" s="26"/>
-      <c r="AH43" s="26"/>
-      <c r="AI43" s="26"/>
-      <c r="AJ43" s="26"/>
-      <c r="AK43" s="26"/>
-      <c r="AL43" s="26"/>
+      <c r="AG43" s="27"/>
+      <c r="AH43" s="27"/>
+      <c r="AI43" s="27"/>
+      <c r="AJ43" s="27"/>
+      <c r="AK43" s="27"/>
+      <c r="AL43" s="27"/>
     </row>
     <row r="44" ht="14.25" customHeight="1">
-      <c r="A44" s="28" t="s">
-        <v>123</v>
-      </c>
-      <c r="B44" s="28" t="s">
-        <v>244</v>
-      </c>
-      <c r="C44" s="9"/>
-      <c r="D44" s="9"/>
-      <c r="E44" s="9"/>
-      <c r="F44" s="9"/>
+      <c r="A44" s="35" t="s">
+        <v>130</v>
+      </c>
+      <c r="B44" s="35" t="s">
+        <v>252</v>
+      </c>
+      <c r="C44" s="30" t="s">
+        <v>41</v>
+      </c>
+      <c r="D44" s="36"/>
+      <c r="E44" s="36"/>
+      <c r="F44" s="30"/>
       <c r="G44" s="9"/>
       <c r="H44" s="9"/>
       <c r="I44" s="9"/>
@@ -3385,8 +3457,8 @@
       <c r="K44" s="9"/>
       <c r="L44" s="9"/>
       <c r="M44" s="9"/>
-      <c r="N44" s="9" t="s">
-        <v>245</v>
+      <c r="N44" s="30" t="s">
+        <v>253</v>
       </c>
       <c r="O44" s="9"/>
       <c r="P44" s="9"/>
@@ -3406,22 +3478,26 @@
       <c r="AD44" s="9"/>
       <c r="AE44" s="9"/>
       <c r="AF44" s="9"/>
-      <c r="AG44" s="26"/>
-      <c r="AH44" s="26"/>
-      <c r="AI44" s="26"/>
-      <c r="AJ44" s="26"/>
-      <c r="AK44" s="26"/>
-      <c r="AL44" s="26"/>
+      <c r="AG44" s="27"/>
+      <c r="AH44" s="27"/>
+      <c r="AI44" s="27"/>
+      <c r="AJ44" s="27"/>
+      <c r="AK44" s="27"/>
+      <c r="AL44" s="27"/>
     </row>
     <row r="45" ht="14.25" customHeight="1">
-      <c r="A45" s="28" t="s">
-        <v>106</v>
-      </c>
-      <c r="B45" s="28"/>
-      <c r="C45" s="9"/>
-      <c r="D45" s="9"/>
-      <c r="E45" s="9"/>
-      <c r="F45" s="9"/>
+      <c r="A45" s="35" t="s">
+        <v>130</v>
+      </c>
+      <c r="B45" s="35" t="s">
+        <v>254</v>
+      </c>
+      <c r="C45" s="30" t="s">
+        <v>41</v>
+      </c>
+      <c r="D45" s="36"/>
+      <c r="E45" s="36"/>
+      <c r="F45" s="30"/>
       <c r="G45" s="9"/>
       <c r="H45" s="9"/>
       <c r="I45" s="9"/>
@@ -3429,7 +3505,9 @@
       <c r="K45" s="9"/>
       <c r="L45" s="9"/>
       <c r="M45" s="9"/>
-      <c r="N45" s="9"/>
+      <c r="N45" s="30" t="s">
+        <v>255</v>
+      </c>
       <c r="O45" s="9"/>
       <c r="P45" s="9"/>
       <c r="Q45" s="9"/>
@@ -3448,34 +3526,32 @@
       <c r="AD45" s="9"/>
       <c r="AE45" s="9"/>
       <c r="AF45" s="9"/>
-      <c r="AG45" s="26"/>
-      <c r="AH45" s="26"/>
-      <c r="AI45" s="26"/>
-      <c r="AJ45" s="26"/>
-      <c r="AK45" s="26"/>
-      <c r="AL45" s="26"/>
+      <c r="AG45" s="27"/>
+      <c r="AH45" s="27"/>
+      <c r="AI45" s="27"/>
+      <c r="AJ45" s="27"/>
+      <c r="AK45" s="27"/>
+      <c r="AL45" s="27"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
-      <c r="A46" s="28" t="s">
-        <v>33</v>
-      </c>
-      <c r="B46" s="28" t="s">
-        <v>246</v>
+      <c r="A46" s="29" t="s">
+        <v>66</v>
+      </c>
+      <c r="B46" s="29" t="s">
+        <v>256</v>
       </c>
       <c r="C46" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="D46" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="E46" s="29" t="s">
-        <v>42</v>
+        <v>257</v>
+      </c>
+      <c r="D46" s="30" t="s">
+        <v>258</v>
+      </c>
+      <c r="E46" s="30" t="s">
+        <v>259</v>
       </c>
       <c r="F46" s="9"/>
       <c r="G46" s="9"/>
-      <c r="H46" s="9" t="s">
-        <v>92</v>
-      </c>
+      <c r="H46" s="9"/>
       <c r="I46" s="9"/>
       <c r="J46" s="9"/>
       <c r="K46" s="9"/>
@@ -3500,34 +3576,40 @@
       <c r="AD46" s="9"/>
       <c r="AE46" s="9"/>
       <c r="AF46" s="9"/>
-      <c r="AG46" s="26"/>
-      <c r="AH46" s="26"/>
-      <c r="AI46" s="26"/>
-      <c r="AJ46" s="26"/>
-      <c r="AK46" s="26"/>
-      <c r="AL46" s="26"/>
+      <c r="AG46" s="27"/>
+      <c r="AH46" s="27"/>
+      <c r="AI46" s="27"/>
+      <c r="AJ46" s="27"/>
+      <c r="AK46" s="27"/>
+      <c r="AL46" s="27"/>
     </row>
     <row r="47" ht="14.25" customHeight="1">
-      <c r="A47" s="28" t="s">
-        <v>123</v>
-      </c>
-      <c r="B47" s="28" t="s">
-        <v>247</v>
-      </c>
-      <c r="C47" s="9"/>
-      <c r="D47" s="9"/>
-      <c r="E47" s="9"/>
+      <c r="A47" s="29" t="s">
+        <v>66</v>
+      </c>
+      <c r="B47" s="29" t="s">
+        <v>260</v>
+      </c>
+      <c r="C47" s="9" t="s">
+        <v>261</v>
+      </c>
+      <c r="D47" s="30" t="s">
+        <v>261</v>
+      </c>
+      <c r="E47" s="30" t="s">
+        <v>262</v>
+      </c>
       <c r="F47" s="9"/>
       <c r="G47" s="9"/>
-      <c r="H47" s="9"/>
+      <c r="H47" s="9" t="s">
+        <v>263</v>
+      </c>
       <c r="I47" s="9"/>
       <c r="J47" s="9"/>
       <c r="K47" s="9"/>
       <c r="L47" s="9"/>
       <c r="M47" s="9"/>
-      <c r="N47" s="9" t="s">
-        <v>248</v>
-      </c>
+      <c r="N47" s="9"/>
       <c r="O47" s="9"/>
       <c r="P47" s="9"/>
       <c r="Q47" s="9"/>
@@ -3546,23 +3628,29 @@
       <c r="AD47" s="9"/>
       <c r="AE47" s="9"/>
       <c r="AF47" s="9"/>
-      <c r="AG47" s="26"/>
-      <c r="AH47" s="26"/>
-      <c r="AI47" s="26"/>
-      <c r="AJ47" s="26"/>
-      <c r="AK47" s="26"/>
-      <c r="AL47" s="26"/>
+      <c r="AG47" s="27"/>
+      <c r="AH47" s="27"/>
+      <c r="AI47" s="27"/>
+      <c r="AJ47" s="27"/>
+      <c r="AK47" s="27"/>
+      <c r="AL47" s="27"/>
     </row>
     <row r="48" ht="14.25" customHeight="1">
-      <c r="A48" s="28" t="s">
-        <v>123</v>
-      </c>
-      <c r="B48" s="28" t="s">
-        <v>249</v>
-      </c>
-      <c r="C48" s="9"/>
-      <c r="D48" s="9"/>
-      <c r="E48" s="9"/>
+      <c r="A48" s="29" t="s">
+        <v>33</v>
+      </c>
+      <c r="B48" s="29" t="s">
+        <v>264</v>
+      </c>
+      <c r="C48" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="D48" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="E48" s="30" t="s">
+        <v>41</v>
+      </c>
       <c r="F48" s="9"/>
       <c r="G48" s="9"/>
       <c r="H48" s="9"/>
@@ -3571,9 +3659,7 @@
       <c r="K48" s="9"/>
       <c r="L48" s="9"/>
       <c r="M48" s="9"/>
-      <c r="N48" s="9" t="s">
-        <v>250</v>
-      </c>
+      <c r="N48" s="9"/>
       <c r="O48" s="9"/>
       <c r="P48" s="9"/>
       <c r="Q48" s="9"/>
@@ -3592,19 +3678,19 @@
       <c r="AD48" s="9"/>
       <c r="AE48" s="9"/>
       <c r="AF48" s="9"/>
-      <c r="AG48" s="26"/>
-      <c r="AH48" s="26"/>
-      <c r="AI48" s="26"/>
-      <c r="AJ48" s="26"/>
-      <c r="AK48" s="26"/>
-      <c r="AL48" s="26"/>
+      <c r="AG48" s="27"/>
+      <c r="AH48" s="27"/>
+      <c r="AI48" s="27"/>
+      <c r="AJ48" s="27"/>
+      <c r="AK48" s="27"/>
+      <c r="AL48" s="27"/>
     </row>
     <row r="49" ht="14.25" customHeight="1">
-      <c r="A49" s="28" t="s">
-        <v>123</v>
-      </c>
-      <c r="B49" s="28" t="s">
-        <v>251</v>
+      <c r="A49" s="29" t="s">
+        <v>130</v>
+      </c>
+      <c r="B49" s="29" t="s">
+        <v>265</v>
       </c>
       <c r="C49" s="9"/>
       <c r="D49" s="9"/>
@@ -3618,7 +3704,7 @@
       <c r="L49" s="9"/>
       <c r="M49" s="9"/>
       <c r="N49" s="9" t="s">
-        <v>252</v>
+        <v>266</v>
       </c>
       <c r="O49" s="9"/>
       <c r="P49" s="9"/>
@@ -3638,18 +3724,18 @@
       <c r="AD49" s="9"/>
       <c r="AE49" s="9"/>
       <c r="AF49" s="9"/>
-      <c r="AG49" s="26"/>
-      <c r="AH49" s="26"/>
-      <c r="AI49" s="26"/>
-      <c r="AJ49" s="26"/>
-      <c r="AK49" s="26"/>
-      <c r="AL49" s="26"/>
+      <c r="AG49" s="27"/>
+      <c r="AH49" s="27"/>
+      <c r="AI49" s="27"/>
+      <c r="AJ49" s="27"/>
+      <c r="AK49" s="27"/>
+      <c r="AL49" s="27"/>
     </row>
     <row r="50" ht="14.25" customHeight="1">
-      <c r="A50" s="28" t="s">
-        <v>106</v>
-      </c>
-      <c r="B50" s="28"/>
+      <c r="A50" s="29" t="s">
+        <v>88</v>
+      </c>
+      <c r="B50" s="29"/>
       <c r="C50" s="9"/>
       <c r="D50" s="9"/>
       <c r="E50" s="9"/>
@@ -3680,24 +3766,34 @@
       <c r="AD50" s="9"/>
       <c r="AE50" s="9"/>
       <c r="AF50" s="9"/>
-      <c r="AG50" s="26"/>
-      <c r="AH50" s="26"/>
-      <c r="AI50" s="26"/>
-      <c r="AJ50" s="26"/>
-      <c r="AK50" s="26"/>
-      <c r="AL50" s="26"/>
+      <c r="AG50" s="27"/>
+      <c r="AH50" s="27"/>
+      <c r="AI50" s="27"/>
+      <c r="AJ50" s="27"/>
+      <c r="AK50" s="27"/>
+      <c r="AL50" s="27"/>
     </row>
     <row r="51" ht="14.25" customHeight="1">
-      <c r="A51" s="28" t="s">
-        <v>106</v>
-      </c>
-      <c r="B51" s="28"/>
-      <c r="C51" s="9"/>
-      <c r="D51" s="9"/>
-      <c r="E51" s="9"/>
+      <c r="A51" s="29" t="s">
+        <v>33</v>
+      </c>
+      <c r="B51" s="29" t="s">
+        <v>267</v>
+      </c>
+      <c r="C51" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="D51" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="E51" s="30" t="s">
+        <v>41</v>
+      </c>
       <c r="F51" s="9"/>
       <c r="G51" s="9"/>
-      <c r="H51" s="9"/>
+      <c r="H51" s="9" t="s">
+        <v>87</v>
+      </c>
       <c r="I51" s="9"/>
       <c r="J51" s="9"/>
       <c r="K51" s="9"/>
@@ -3722,18 +3818,235 @@
       <c r="AD51" s="9"/>
       <c r="AE51" s="9"/>
       <c r="AF51" s="9"/>
-      <c r="AG51" s="26"/>
-      <c r="AH51" s="26"/>
-      <c r="AI51" s="26"/>
-      <c r="AJ51" s="26"/>
-      <c r="AK51" s="26"/>
-      <c r="AL51" s="26"/>
-    </row>
-    <row r="52" ht="14.25" customHeight="1"/>
-    <row r="53" ht="14.25" customHeight="1"/>
-    <row r="54" ht="14.25" customHeight="1"/>
-    <row r="55" ht="14.25" customHeight="1"/>
-    <row r="56" ht="14.25" customHeight="1"/>
+      <c r="AG51" s="27"/>
+      <c r="AH51" s="27"/>
+      <c r="AI51" s="27"/>
+      <c r="AJ51" s="27"/>
+      <c r="AK51" s="27"/>
+      <c r="AL51" s="27"/>
+    </row>
+    <row r="52" ht="14.25" customHeight="1">
+      <c r="A52" s="29" t="s">
+        <v>130</v>
+      </c>
+      <c r="B52" s="29" t="s">
+        <v>268</v>
+      </c>
+      <c r="C52" s="9"/>
+      <c r="D52" s="9"/>
+      <c r="E52" s="9"/>
+      <c r="F52" s="9"/>
+      <c r="G52" s="9"/>
+      <c r="H52" s="9"/>
+      <c r="I52" s="9"/>
+      <c r="J52" s="9"/>
+      <c r="K52" s="9"/>
+      <c r="L52" s="9"/>
+      <c r="M52" s="9"/>
+      <c r="N52" s="9" t="s">
+        <v>269</v>
+      </c>
+      <c r="O52" s="9"/>
+      <c r="P52" s="9"/>
+      <c r="Q52" s="9"/>
+      <c r="R52" s="9"/>
+      <c r="S52" s="9"/>
+      <c r="T52" s="9"/>
+      <c r="U52" s="9"/>
+      <c r="V52" s="9"/>
+      <c r="W52" s="9"/>
+      <c r="X52" s="9"/>
+      <c r="Y52" s="9"/>
+      <c r="Z52" s="9"/>
+      <c r="AA52" s="9"/>
+      <c r="AB52" s="9"/>
+      <c r="AC52" s="9"/>
+      <c r="AD52" s="9"/>
+      <c r="AE52" s="9"/>
+      <c r="AF52" s="9"/>
+      <c r="AG52" s="27"/>
+      <c r="AH52" s="27"/>
+      <c r="AI52" s="27"/>
+      <c r="AJ52" s="27"/>
+      <c r="AK52" s="27"/>
+      <c r="AL52" s="27"/>
+    </row>
+    <row r="53" ht="14.25" customHeight="1">
+      <c r="A53" s="29" t="s">
+        <v>130</v>
+      </c>
+      <c r="B53" s="29" t="s">
+        <v>270</v>
+      </c>
+      <c r="C53" s="9"/>
+      <c r="D53" s="9"/>
+      <c r="E53" s="9"/>
+      <c r="F53" s="9"/>
+      <c r="G53" s="9"/>
+      <c r="H53" s="9"/>
+      <c r="I53" s="9"/>
+      <c r="J53" s="9"/>
+      <c r="K53" s="9"/>
+      <c r="L53" s="9"/>
+      <c r="M53" s="9"/>
+      <c r="N53" s="9" t="s">
+        <v>271</v>
+      </c>
+      <c r="O53" s="9"/>
+      <c r="P53" s="9"/>
+      <c r="Q53" s="9"/>
+      <c r="R53" s="9"/>
+      <c r="S53" s="9"/>
+      <c r="T53" s="9"/>
+      <c r="U53" s="9"/>
+      <c r="V53" s="9"/>
+      <c r="W53" s="9"/>
+      <c r="X53" s="9"/>
+      <c r="Y53" s="9"/>
+      <c r="Z53" s="9"/>
+      <c r="AA53" s="9"/>
+      <c r="AB53" s="9"/>
+      <c r="AC53" s="9"/>
+      <c r="AD53" s="9"/>
+      <c r="AE53" s="9"/>
+      <c r="AF53" s="9"/>
+      <c r="AG53" s="27"/>
+      <c r="AH53" s="27"/>
+      <c r="AI53" s="27"/>
+      <c r="AJ53" s="27"/>
+      <c r="AK53" s="27"/>
+      <c r="AL53" s="27"/>
+    </row>
+    <row r="54" ht="14.25" customHeight="1">
+      <c r="A54" s="29" t="s">
+        <v>130</v>
+      </c>
+      <c r="B54" s="29" t="s">
+        <v>272</v>
+      </c>
+      <c r="C54" s="9"/>
+      <c r="D54" s="9"/>
+      <c r="E54" s="9"/>
+      <c r="F54" s="9"/>
+      <c r="G54" s="9"/>
+      <c r="H54" s="9"/>
+      <c r="I54" s="9"/>
+      <c r="J54" s="9"/>
+      <c r="K54" s="9"/>
+      <c r="L54" s="9"/>
+      <c r="M54" s="9"/>
+      <c r="N54" s="9" t="s">
+        <v>273</v>
+      </c>
+      <c r="O54" s="9"/>
+      <c r="P54" s="9"/>
+      <c r="Q54" s="9"/>
+      <c r="R54" s="9"/>
+      <c r="S54" s="9"/>
+      <c r="T54" s="9"/>
+      <c r="U54" s="9"/>
+      <c r="V54" s="9"/>
+      <c r="W54" s="9"/>
+      <c r="X54" s="9"/>
+      <c r="Y54" s="9"/>
+      <c r="Z54" s="9"/>
+      <c r="AA54" s="9"/>
+      <c r="AB54" s="9"/>
+      <c r="AC54" s="9"/>
+      <c r="AD54" s="9"/>
+      <c r="AE54" s="9"/>
+      <c r="AF54" s="9"/>
+      <c r="AG54" s="27"/>
+      <c r="AH54" s="27"/>
+      <c r="AI54" s="27"/>
+      <c r="AJ54" s="27"/>
+      <c r="AK54" s="27"/>
+      <c r="AL54" s="27"/>
+    </row>
+    <row r="55" ht="14.25" customHeight="1">
+      <c r="A55" s="29" t="s">
+        <v>88</v>
+      </c>
+      <c r="B55" s="29"/>
+      <c r="C55" s="9"/>
+      <c r="D55" s="9"/>
+      <c r="E55" s="9"/>
+      <c r="F55" s="9"/>
+      <c r="G55" s="9"/>
+      <c r="H55" s="9"/>
+      <c r="I55" s="9"/>
+      <c r="J55" s="9"/>
+      <c r="K55" s="9"/>
+      <c r="L55" s="9"/>
+      <c r="M55" s="9"/>
+      <c r="N55" s="9"/>
+      <c r="O55" s="9"/>
+      <c r="P55" s="9"/>
+      <c r="Q55" s="9"/>
+      <c r="R55" s="9"/>
+      <c r="S55" s="9"/>
+      <c r="T55" s="9"/>
+      <c r="U55" s="9"/>
+      <c r="V55" s="9"/>
+      <c r="W55" s="9"/>
+      <c r="X55" s="9"/>
+      <c r="Y55" s="9"/>
+      <c r="Z55" s="9"/>
+      <c r="AA55" s="9"/>
+      <c r="AB55" s="9"/>
+      <c r="AC55" s="9"/>
+      <c r="AD55" s="9"/>
+      <c r="AE55" s="9"/>
+      <c r="AF55" s="9"/>
+      <c r="AG55" s="27"/>
+      <c r="AH55" s="27"/>
+      <c r="AI55" s="27"/>
+      <c r="AJ55" s="27"/>
+      <c r="AK55" s="27"/>
+      <c r="AL55" s="27"/>
+    </row>
+    <row r="56" ht="14.25" customHeight="1">
+      <c r="A56" s="29" t="s">
+        <v>88</v>
+      </c>
+      <c r="B56" s="29"/>
+      <c r="C56" s="9"/>
+      <c r="D56" s="9"/>
+      <c r="E56" s="9"/>
+      <c r="F56" s="9"/>
+      <c r="G56" s="9"/>
+      <c r="H56" s="9"/>
+      <c r="I56" s="9"/>
+      <c r="J56" s="9"/>
+      <c r="K56" s="9"/>
+      <c r="L56" s="9"/>
+      <c r="M56" s="9"/>
+      <c r="N56" s="9"/>
+      <c r="O56" s="9"/>
+      <c r="P56" s="9"/>
+      <c r="Q56" s="9"/>
+      <c r="R56" s="9"/>
+      <c r="S56" s="9"/>
+      <c r="T56" s="9"/>
+      <c r="U56" s="9"/>
+      <c r="V56" s="9"/>
+      <c r="W56" s="9"/>
+      <c r="X56" s="9"/>
+      <c r="Y56" s="9"/>
+      <c r="Z56" s="9"/>
+      <c r="AA56" s="9"/>
+      <c r="AB56" s="9"/>
+      <c r="AC56" s="9"/>
+      <c r="AD56" s="9"/>
+      <c r="AE56" s="9"/>
+      <c r="AF56" s="9"/>
+      <c r="AG56" s="27"/>
+      <c r="AH56" s="27"/>
+      <c r="AI56" s="27"/>
+      <c r="AJ56" s="27"/>
+      <c r="AK56" s="27"/>
+      <c r="AL56" s="27"/>
+    </row>
     <row r="57" ht="14.25" customHeight="1"/>
     <row r="58" ht="14.25" customHeight="1"/>
     <row r="59" ht="14.25" customHeight="1"/>
@@ -4679,6 +4992,11 @@
     <row r="999" ht="14.25" customHeight="1"/>
     <row r="1000" ht="14.25" customHeight="1"/>
     <row r="1001" ht="14.25" customHeight="1"/>
+    <row r="1002" ht="14.25" customHeight="1"/>
+    <row r="1003" ht="14.25" customHeight="1"/>
+    <row r="1004" ht="14.25" customHeight="1"/>
+    <row r="1005" ht="14.25" customHeight="1"/>
+    <row r="1006" ht="14.25" customHeight="1"/>
   </sheetData>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
@@ -4702,399 +5020,489 @@
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
-      <c r="A1" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="4" t="s">
+      <c r="A1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="B1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="C1" s="2" t="s">
         <v>5</v>
       </c>
+      <c r="D1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
-      <c r="A2" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="B2" s="8" t="s">
+      <c r="A2" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="D2" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="C2" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="D2" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="E2" s="7" t="s">
+      <c r="E2" s="6" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
-      <c r="A3" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="B3" s="8" t="s">
+      <c r="A3" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="7" t="s">
         <v>35</v>
       </c>
       <c r="D3" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="6" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="4" ht="14.25" customHeight="1">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="7" t="s">
         <v>40</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>43</v>
+        <v>42</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>45</v>
+      <c r="B5" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>47</v>
       </c>
       <c r="D5" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" ht="14.25" customHeight="1">
+      <c r="A6" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="7" ht="14.25" customHeight="1">
+      <c r="A7" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B7" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="E5" s="7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="6" ht="14.25" customHeight="1">
-      <c r="A6" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="7" ht="14.25" customHeight="1">
-      <c r="A7" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>52</v>
+      <c r="C7" s="7" t="s">
+        <v>55</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>54</v>
+        <v>56</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
-      <c r="A8" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="B8" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="C8" s="15" t="s">
+      <c r="A8" s="4" t="s">
         <v>58</v>
       </c>
+      <c r="B8" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="C8" s="16" t="s">
+        <v>61</v>
+      </c>
       <c r="D8" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>60</v>
+        <v>62</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
-      <c r="A9" s="16" t="s">
-        <v>63</v>
-      </c>
-      <c r="B9" s="17" t="s">
+      <c r="A9" s="17" t="s">
         <v>64</v>
       </c>
+      <c r="B9" s="18" t="s">
+        <v>65</v>
+      </c>
       <c r="C9" s="19" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="D9" s="20" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>68</v>
-      </c>
-      <c r="F9" s="16"/>
-      <c r="G9" s="16"/>
-      <c r="H9" s="16"/>
-      <c r="I9" s="16"/>
-      <c r="J9" s="16"/>
-      <c r="K9" s="16"/>
-      <c r="L9" s="16"/>
-      <c r="M9" s="16"/>
-      <c r="N9" s="16"/>
-      <c r="O9" s="16"/>
-      <c r="P9" s="16"/>
-      <c r="Q9" s="16"/>
-      <c r="R9" s="16"/>
-      <c r="S9" s="16"/>
-      <c r="T9" s="16"/>
-      <c r="U9" s="16"/>
+        <v>73</v>
+      </c>
+      <c r="F9" s="17"/>
+      <c r="G9" s="17"/>
+      <c r="H9" s="17"/>
+      <c r="I9" s="17"/>
+      <c r="J9" s="17"/>
+      <c r="K9" s="17"/>
+      <c r="L9" s="17"/>
+      <c r="M9" s="17"/>
+      <c r="N9" s="17"/>
+      <c r="O9" s="17"/>
+      <c r="P9" s="17"/>
+      <c r="Q9" s="17"/>
+      <c r="R9" s="17"/>
+      <c r="S9" s="17"/>
+      <c r="T9" s="17"/>
+      <c r="U9" s="17"/>
     </row>
     <row r="10" ht="14.25" customHeight="1">
-      <c r="A10" s="16" t="s">
-        <v>63</v>
-      </c>
-      <c r="B10" s="17" t="s">
-        <v>71</v>
+      <c r="A10" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="B10" s="18" t="s">
+        <v>78</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="D10" s="20" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>77</v>
-      </c>
-      <c r="F10" s="16"/>
-      <c r="G10" s="16"/>
-      <c r="H10" s="16"/>
-      <c r="I10" s="16"/>
-      <c r="J10" s="16"/>
-      <c r="K10" s="16"/>
-      <c r="L10" s="16"/>
-      <c r="M10" s="16"/>
-      <c r="N10" s="16"/>
-      <c r="O10" s="16"/>
-      <c r="P10" s="16"/>
-      <c r="Q10" s="16"/>
-      <c r="R10" s="16"/>
-      <c r="S10" s="16"/>
-      <c r="T10" s="16"/>
-      <c r="U10" s="16"/>
+        <v>81</v>
+      </c>
+      <c r="F10" s="17"/>
+      <c r="G10" s="17"/>
+      <c r="H10" s="17"/>
+      <c r="I10" s="17"/>
+      <c r="J10" s="17"/>
+      <c r="K10" s="17"/>
+      <c r="L10" s="17"/>
+      <c r="M10" s="17"/>
+      <c r="N10" s="17"/>
+      <c r="O10" s="17"/>
+      <c r="P10" s="17"/>
+      <c r="Q10" s="17"/>
+      <c r="R10" s="17"/>
+      <c r="S10" s="17"/>
+      <c r="T10" s="17"/>
+      <c r="U10" s="17"/>
     </row>
     <row r="11" ht="14.25" customHeight="1">
-      <c r="A11" s="16" t="s">
-        <v>63</v>
-      </c>
-      <c r="B11" s="17" t="s">
-        <v>78</v>
+      <c r="A11" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="B11" s="18" t="s">
+        <v>85</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="D11" s="20" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("GOOGLETRANSLATE(C11, ""en"", ""fr"")"),"Entrepreneur en santé communautaire")</f>
         <v>Entrepreneur en santé communautaire</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>87</v>
-      </c>
-      <c r="F11" s="16"/>
-      <c r="G11" s="16"/>
-      <c r="H11" s="16"/>
-      <c r="I11" s="16"/>
-      <c r="J11" s="16"/>
-      <c r="K11" s="16"/>
-      <c r="L11" s="16"/>
-      <c r="M11" s="16"/>
-      <c r="N11" s="16"/>
-      <c r="O11" s="16"/>
-      <c r="P11" s="16"/>
-      <c r="Q11" s="16"/>
-      <c r="R11" s="16"/>
-      <c r="S11" s="16"/>
-      <c r="T11" s="16"/>
-      <c r="U11" s="16"/>
+        <v>89</v>
+      </c>
+      <c r="F11" s="17"/>
+      <c r="G11" s="17"/>
+      <c r="H11" s="17"/>
+      <c r="I11" s="17"/>
+      <c r="J11" s="17"/>
+      <c r="K11" s="17"/>
+      <c r="L11" s="17"/>
+      <c r="M11" s="17"/>
+      <c r="N11" s="17"/>
+      <c r="O11" s="17"/>
+      <c r="P11" s="17"/>
+      <c r="Q11" s="17"/>
+      <c r="R11" s="17"/>
+      <c r="S11" s="17"/>
+      <c r="T11" s="17"/>
+      <c r="U11" s="17"/>
     </row>
     <row r="12" ht="14.25" customHeight="1">
-      <c r="A12" s="16" t="s">
-        <v>63</v>
-      </c>
-      <c r="B12" s="17" t="s">
-        <v>88</v>
+      <c r="A12" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="B12" s="18" t="s">
+        <v>90</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D12" s="20" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E12" s="21" t="s">
-        <v>91</v>
-      </c>
-      <c r="F12" s="16"/>
-      <c r="G12" s="16"/>
-      <c r="H12" s="16"/>
-      <c r="I12" s="16"/>
-      <c r="J12" s="16"/>
-      <c r="K12" s="16"/>
-      <c r="L12" s="16"/>
-      <c r="M12" s="16"/>
-      <c r="N12" s="16"/>
-      <c r="O12" s="16"/>
-      <c r="P12" s="16"/>
-      <c r="Q12" s="16"/>
-      <c r="R12" s="16"/>
-      <c r="S12" s="16"/>
-      <c r="T12" s="16"/>
-      <c r="U12" s="16"/>
+        <v>93</v>
+      </c>
+      <c r="F12" s="17"/>
+      <c r="G12" s="17"/>
+      <c r="H12" s="17"/>
+      <c r="I12" s="17"/>
+      <c r="J12" s="17"/>
+      <c r="K12" s="17"/>
+      <c r="L12" s="17"/>
+      <c r="M12" s="17"/>
+      <c r="N12" s="17"/>
+      <c r="O12" s="17"/>
+      <c r="P12" s="17"/>
+      <c r="Q12" s="17"/>
+      <c r="R12" s="17"/>
+      <c r="S12" s="17"/>
+      <c r="T12" s="17"/>
+      <c r="U12" s="17"/>
     </row>
     <row r="13" ht="14.25" customHeight="1">
-      <c r="A13" s="16" t="s">
-        <v>63</v>
-      </c>
-      <c r="B13" s="16" t="s">
-        <v>93</v>
-      </c>
-      <c r="C13" s="16" t="s">
+      <c r="A13" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="B13" s="17" t="s">
         <v>94</v>
       </c>
+      <c r="C13" s="17" t="s">
+        <v>95</v>
+      </c>
       <c r="D13" s="20" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E13" s="21" t="s">
-        <v>95</v>
-      </c>
-      <c r="F13" s="16"/>
-      <c r="G13" s="16"/>
-      <c r="H13" s="16"/>
-      <c r="I13" s="16"/>
-      <c r="J13" s="16"/>
-      <c r="K13" s="16"/>
-      <c r="L13" s="16"/>
-      <c r="M13" s="16"/>
-      <c r="N13" s="16"/>
-      <c r="O13" s="16"/>
-      <c r="P13" s="16"/>
-      <c r="Q13" s="16"/>
-      <c r="R13" s="16"/>
-      <c r="S13" s="16"/>
-      <c r="T13" s="16"/>
-      <c r="U13" s="16"/>
+        <v>96</v>
+      </c>
+      <c r="F13" s="17"/>
+      <c r="G13" s="17"/>
+      <c r="H13" s="17"/>
+      <c r="I13" s="17"/>
+      <c r="J13" s="17"/>
+      <c r="K13" s="17"/>
+      <c r="L13" s="17"/>
+      <c r="M13" s="17"/>
+      <c r="N13" s="17"/>
+      <c r="O13" s="17"/>
+      <c r="P13" s="17"/>
+      <c r="Q13" s="17"/>
+      <c r="R13" s="17"/>
+      <c r="S13" s="17"/>
+      <c r="T13" s="17"/>
+      <c r="U13" s="17"/>
     </row>
     <row r="14" ht="14.25" customHeight="1">
-      <c r="A14" s="16" t="s">
-        <v>63</v>
-      </c>
-      <c r="B14" s="17" t="s">
-        <v>96</v>
+      <c r="A14" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="B14" s="18" t="s">
+        <v>98</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D14" s="20" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E14" s="21" t="s">
-        <v>99</v>
-      </c>
-      <c r="F14" s="16"/>
-      <c r="G14" s="16"/>
-      <c r="H14" s="16"/>
-      <c r="I14" s="16"/>
-      <c r="J14" s="16"/>
-      <c r="K14" s="16"/>
-      <c r="L14" s="16"/>
-      <c r="M14" s="16"/>
-      <c r="N14" s="16"/>
-      <c r="O14" s="16"/>
-      <c r="P14" s="16"/>
-      <c r="Q14" s="16"/>
-      <c r="R14" s="16"/>
-      <c r="S14" s="16"/>
-      <c r="T14" s="16"/>
-      <c r="U14" s="16"/>
+        <v>101</v>
+      </c>
+      <c r="F14" s="17"/>
+      <c r="G14" s="17"/>
+      <c r="H14" s="17"/>
+      <c r="I14" s="17"/>
+      <c r="J14" s="17"/>
+      <c r="K14" s="17"/>
+      <c r="L14" s="17"/>
+      <c r="M14" s="17"/>
+      <c r="N14" s="17"/>
+      <c r="O14" s="17"/>
+      <c r="P14" s="17"/>
+      <c r="Q14" s="17"/>
+      <c r="R14" s="17"/>
+      <c r="S14" s="17"/>
+      <c r="T14" s="17"/>
+      <c r="U14" s="17"/>
     </row>
     <row r="15" ht="14.25" customHeight="1">
-      <c r="A15" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="B15" s="13" t="s">
-        <v>101</v>
+      <c r="A15" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B15" s="15" t="s">
+        <v>104</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="D15" s="20" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("GOOGLETRANSLATE(C15, ""en"", ""fr"")"),"Département du pays")</f>
         <v>Département du pays</v>
       </c>
-      <c r="E15" s="7" t="s">
+      <c r="E15" s="6" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="16" ht="14.25" customHeight="1">
+      <c r="A16" s="4" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="16" ht="14.25" customHeight="1">
-      <c r="A16" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="B16" s="13" t="s">
-        <v>104</v>
+      <c r="B16" s="15" t="s">
+        <v>114</v>
       </c>
       <c r="C16" s="19" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="D16" s="20" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("GOOGLETRANSLATE(C16, ""en"", ""fr"")"),"Région de supervision")</f>
         <v>Région de supervision</v>
       </c>
-      <c r="E16" s="7" t="s">
-        <v>107</v>
+      <c r="E16" s="6" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
-      <c r="A17" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="B17" s="13" t="s">
-        <v>108</v>
+      <c r="A17" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B17" s="15" t="s">
+        <v>117</v>
       </c>
       <c r="C17" s="19" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="D17" s="20" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("GOOGLETRANSLATE(C17, ""en"", ""fr"")"),"Zone infirmière")</f>
         <v>Zone infirmière</v>
       </c>
-      <c r="E17" s="7" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="18" ht="14.25" customHeight="1"/>
-    <row r="19" ht="14.25" customHeight="1"/>
-    <row r="20" ht="14.25" customHeight="1"/>
-    <row r="21" ht="14.25" customHeight="1"/>
-    <row r="22" ht="14.25" customHeight="1"/>
+      <c r="E17" s="6" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="18" ht="14.25" customHeight="1">
+      <c r="A18" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="D18" s="20" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("GOOGLETRANSLATE(C18, ""en"", ""fr"")"),"Hypertension")</f>
+        <v>Hypertension</v>
+      </c>
+      <c r="E18" s="25" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("GOOGLETRANSLATE(C18, ""en"", ""ht"")"),"Ipètansyon")</f>
+        <v>Ipètansyon</v>
+      </c>
+    </row>
+    <row r="19" ht="14.25" customHeight="1">
+      <c r="A19" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="D19" s="20" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("GOOGLETRANSLATE(C19, ""en"", ""fr"")"),"Diabète")</f>
+        <v>Diabète</v>
+      </c>
+      <c r="E19" s="25" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("GOOGLETRANSLATE(C19, ""en"", ""ht"")"),"Dyabèt")</f>
+        <v>Dyabèt</v>
+      </c>
+    </row>
+    <row r="20" ht="14.25" customHeight="1">
+      <c r="A20" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="D20" s="20" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("GOOGLETRANSLATE(C20, ""en"", ""fr"")"),"AVC antérieur")</f>
+        <v>AVC antérieur</v>
+      </c>
+      <c r="E20" s="25" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("GOOGLETRANSLATE(C20, ""en"", ""ht"")"),"Konjesyon serebral anvan an")</f>
+        <v>Konjesyon serebral anvan an</v>
+      </c>
+    </row>
+    <row r="21" ht="14.25" customHeight="1">
+      <c r="A21" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="D21" s="20" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("GOOGLETRANSLATE(C21, ""en"", ""fr"")"),"Asthme")</f>
+        <v>Asthme</v>
+      </c>
+      <c r="E21" s="25" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("GOOGLETRANSLATE(C21, ""en"", ""ht"")"),"Asm")</f>
+        <v>Asm</v>
+      </c>
+    </row>
+    <row r="22" ht="14.25" customHeight="1">
+      <c r="A22" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="D22" s="20" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("GOOGLETRANSLATE(C22, ""en"", ""fr"")"),"Aucune des réponses ci-dessus")</f>
+        <v>Aucune des réponses ci-dessus</v>
+      </c>
+      <c r="E22" s="25" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("GOOGLETRANSLATE(C22, ""en"", ""ht"")"),"Okenn nan sa ki anwo yo")</f>
+        <v>Okenn nan sa ki anwo yo</v>
+      </c>
+    </row>
     <row r="23" ht="14.25" customHeight="1"/>
     <row r="24" ht="14.25" customHeight="1"/>
     <row r="25" ht="14.25" customHeight="1"/>
@@ -6088,7 +6496,8 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
-    <col customWidth="1" min="1" max="2" width="7.71"/>
+    <col customWidth="1" min="1" max="1" width="11.71"/>
+    <col customWidth="1" min="2" max="2" width="13.43"/>
     <col customWidth="1" min="3" max="3" width="20.43"/>
     <col customWidth="1" min="4" max="6" width="7.71"/>
     <col customWidth="1" min="7" max="26" width="14.29"/>
@@ -6096,40 +6505,40 @@
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
       <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>10</v>
-      </c>
       <c r="D1" s="1" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" ht="14.25" customHeight="1">
+      <c r="A2" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="2" ht="14.25" customHeight="1">
-      <c r="A2" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C2" s="14" t="str">
+      <c r="C2" s="11" t="str">
         <f>TEXT(NOW(), "yyyy-mm-dd_HH-MM")</f>
-        <v>2026-09-24_00-46</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>62</v>
+        <v>2026-10-11_17-44</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="3" ht="14.25" customHeight="1"/>

</xml_diff>